<commit_message>
Decouple service-level tiers from symposiums: recommendedTier as changeable default, readiness notes, no location-equals-tier identity
</commit_message>
<xml_diff>
--- a/pricing-model.xlsx
+++ b/pricing-model.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="118">
   <si>
     <t xml:space="preserve">AWS 1P Public Sector Symposiums - Pricing Model</t>
   </si>
@@ -282,19 +282,52 @@
     <t xml:space="preserve">tiers[premium].preset</t>
   </si>
   <si>
+    <t xml:space="preserve">Symposium readiness and recommended starting service level</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recommendations only. The client confirmed the events and their readiness; the tier mapping is our suggestion and changeable on the Calculator.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Symposium</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recommended tier</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Readiness (confirmed)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">London</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Content is already written</t>
+  </si>
+  <si>
+    <t xml:space="preserve">symposiums[london].recommendedTier / .readiness</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ottawa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Owner in place; story still needs writing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">symposiums[ottawa].recommendedTier / .readiness</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Canberra</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Starting from scratch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">symposiums[canberra].recommendedTier / .readiness</t>
+  </si>
+  <si>
     <t xml:space="preserve">Per-Deck Pricing Calculator</t>
   </si>
   <si>
-    <t xml:space="preserve">London, Ottawa, and Canberra pull inputs from the tier presets (change the blue tier name, or edit presets on Assumptions). Custom column is free-form. Estimate, not a quote.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">London</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ottawa</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Canberra</t>
+    <t xml:space="preserve">Tiers are service levels, not locations: any symposium can run at any tier. The blue tier name per city defaults to OUR recommended starting point (based on readiness) and is fully changeable. Custom column is free-form. Estimate, not a quote.</t>
   </si>
   <si>
     <t xml:space="preserve">Custom</t>
@@ -488,11 +521,15 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="33">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -509,7 +546,47 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -517,10 +594,6 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -529,22 +602,6 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -573,11 +630,11 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -852,88 +909,88 @@
   <dimension ref="A1:A18"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="110"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="110"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+    <row r="2" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2"/>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="3"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="3" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="2" t="s">
+    <row r="6" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="3" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="2" t="s">
+    <row r="7" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="3" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="2"/>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="3"/>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="4" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="2" t="s">
+    <row r="10" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="3" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="2"/>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="3" t="s">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="3"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="4" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="2" t="s">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="2" t="s">
+    <row r="14" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="3" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="2" t="s">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="3" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="2" t="s">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="3" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="2"/>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="4" t="s">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="3"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="5" t="s">
         <v>13</v>
       </c>
     </row>
@@ -953,571 +1010,637 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H43"/>
+  <dimension ref="A1:H50"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="2" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="5" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="2" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="5" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="30"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="5" t="s">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="6" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="6" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="7" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="7" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="8" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="8" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="B5" s="8" t="s">
+      <c r="B5" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="C5" s="8" t="s">
+      <c r="C5" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="H5" s="8" t="s">
+      <c r="H5" s="9" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="9" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="B6" s="10" t="n">
+      <c r="B6" s="11" t="n">
         <v>185</v>
       </c>
-      <c r="C6" s="9" t="s">
+      <c r="C6" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="H6" s="6" t="s">
+      <c r="H6" s="7" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="9" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="B7" s="10" t="n">
+      <c r="B7" s="11" t="n">
         <v>185</v>
       </c>
-      <c r="C7" s="9" t="s">
+      <c r="C7" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="H7" s="6" t="s">
+      <c r="H7" s="7" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="9" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="B8" s="10" t="n">
+      <c r="B8" s="11" t="n">
         <v>175</v>
       </c>
-      <c r="C8" s="9" t="s">
+      <c r="C8" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="H8" s="6" t="s">
+      <c r="H8" s="7" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="9" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="B9" s="10" t="n">
+      <c r="B9" s="11" t="n">
         <v>200</v>
       </c>
-      <c r="C9" s="9" t="s">
+      <c r="C9" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="H9" s="6" t="s">
+      <c r="H9" s="7" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="9" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="B10" s="10" t="n">
+      <c r="B10" s="11" t="n">
         <v>175</v>
       </c>
-      <c r="C10" s="9" t="s">
+      <c r="C10" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="H10" s="6" t="s">
+      <c r="H10" s="7" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="9" t="s">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="B11" s="10" t="n">
+      <c r="B11" s="11" t="n">
         <v>100</v>
       </c>
-      <c r="C11" s="9" t="s">
+      <c r="C11" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="H11" s="6" t="s">
+      <c r="H11" s="7" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="9" t="s">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="B12" s="10" t="n">
+      <c r="B12" s="11" t="n">
         <v>3500</v>
       </c>
-      <c r="C12" s="9" t="s">
+      <c r="C12" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="H12" s="6" t="s">
+      <c r="H12" s="7" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="9" t="s">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="B13" s="10" t="n">
+      <c r="B13" s="11" t="n">
         <v>250</v>
       </c>
-      <c r="C13" s="9" t="s">
+      <c r="C13" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="H13" s="6" t="s">
+      <c r="H13" s="7" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="7" t="s">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="8" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="6" t="s">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="7" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="11" t="s">
+    <row r="18" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="B18" s="11" t="s">
+      <c r="B18" s="12" t="s">
         <v>42</v>
       </c>
-      <c r="C18" s="11" t="s">
+      <c r="C18" s="12" t="s">
         <v>43</v>
       </c>
-      <c r="D18" s="11" t="s">
+      <c r="D18" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="E18" s="11" t="s">
+      <c r="E18" s="12" t="s">
         <v>45</v>
       </c>
-      <c r="F18" s="11" t="s">
+      <c r="F18" s="12" t="s">
         <v>46</v>
       </c>
-      <c r="G18" s="11" t="s">
+      <c r="G18" s="12" t="s">
         <v>47</v>
       </c>
-      <c r="H18" s="11" t="s">
+      <c r="H18" s="12" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="9" t="s">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="B19" s="12" t="n">
+      <c r="B19" s="13" t="n">
         <v>4</v>
       </c>
-      <c r="C19" s="12" t="n">
+      <c r="C19" s="13" t="n">
         <v>16</v>
       </c>
-      <c r="D19" s="12" t="n">
+      <c r="D19" s="13" t="n">
         <v>28</v>
       </c>
-      <c r="E19" s="13" t="n">
+      <c r="E19" s="14" t="n">
         <f aca="false">B19</f>
         <v>4</v>
       </c>
-      <c r="F19" s="13" t="n">
+      <c r="F19" s="14" t="n">
         <f aca="false">E19+C19</f>
         <v>20</v>
       </c>
-      <c r="G19" s="13" t="n">
+      <c r="G19" s="14" t="n">
         <f aca="false">F19+D19</f>
         <v>48</v>
       </c>
-      <c r="H19" s="6" t="s">
+      <c r="H19" s="7" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="9" t="s">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="B20" s="12" t="n">
+      <c r="B20" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="C20" s="12" t="n">
+      <c r="C20" s="13" t="n">
         <v>8</v>
       </c>
-      <c r="D20" s="12" t="n">
+      <c r="D20" s="13" t="n">
         <v>14</v>
       </c>
-      <c r="E20" s="13" t="n">
+      <c r="E20" s="14" t="n">
         <f aca="false">B20</f>
         <v>0</v>
       </c>
-      <c r="F20" s="13" t="n">
+      <c r="F20" s="14" t="n">
         <f aca="false">E20+C20</f>
         <v>8</v>
       </c>
-      <c r="G20" s="13" t="n">
+      <c r="G20" s="14" t="n">
         <f aca="false">F20+D20</f>
         <v>22</v>
       </c>
-      <c r="H20" s="6" t="s">
+      <c r="H20" s="7" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="9" t="s">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="B21" s="12" t="n">
+      <c r="B21" s="13" t="n">
         <v>20</v>
       </c>
-      <c r="C21" s="12" t="n">
+      <c r="C21" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="D21" s="12" t="n">
+      <c r="D21" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="E21" s="13" t="n">
+      <c r="E21" s="14" t="n">
         <f aca="false">B21</f>
         <v>20</v>
       </c>
-      <c r="F21" s="13" t="n">
+      <c r="F21" s="14" t="n">
         <f aca="false">E21+C21</f>
         <v>20</v>
       </c>
-      <c r="G21" s="13" t="n">
+      <c r="G21" s="14" t="n">
         <f aca="false">F21+D21</f>
         <v>20</v>
       </c>
-      <c r="H21" s="6" t="s">
+      <c r="H21" s="7" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="9" t="s">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="B22" s="12" t="n">
+      <c r="B22" s="13" t="n">
         <v>3</v>
       </c>
-      <c r="C22" s="12" t="n">
+      <c r="C22" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="D22" s="12" t="n">
+      <c r="D22" s="13" t="n">
         <v>5</v>
       </c>
-      <c r="E22" s="13" t="n">
+      <c r="E22" s="14" t="n">
         <f aca="false">B22</f>
         <v>3</v>
       </c>
-      <c r="F22" s="13" t="n">
+      <c r="F22" s="14" t="n">
         <f aca="false">E22+C22</f>
         <v>3</v>
       </c>
-      <c r="G22" s="13" t="n">
+      <c r="G22" s="14" t="n">
         <f aca="false">F22+D22</f>
         <v>8</v>
       </c>
-      <c r="H22" s="6" t="s">
+      <c r="H22" s="7" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="9" t="s">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="B23" s="12" t="n">
+      <c r="B23" s="13" t="n">
         <v>6</v>
       </c>
-      <c r="C23" s="12" t="n">
+      <c r="C23" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="D23" s="12" t="n">
+      <c r="D23" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="E23" s="13" t="n">
+      <c r="E23" s="14" t="n">
         <f aca="false">B23</f>
         <v>6</v>
       </c>
-      <c r="F23" s="13" t="n">
+      <c r="F23" s="14" t="n">
         <f aca="false">E23+C23</f>
         <v>6</v>
       </c>
-      <c r="G23" s="13" t="n">
+      <c r="G23" s="14" t="n">
         <f aca="false">F23+D23</f>
         <v>6</v>
       </c>
-      <c r="H23" s="6" t="s">
+      <c r="H23" s="7" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="9" t="s">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="B24" s="12" t="n">
+      <c r="B24" s="13" t="n">
         <v>5</v>
       </c>
-      <c r="C24" s="12" t="n">
+      <c r="C24" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="D24" s="12" t="n">
+      <c r="D24" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="E24" s="13" t="n">
+      <c r="E24" s="14" t="n">
         <f aca="false">B24</f>
         <v>5</v>
       </c>
-      <c r="F24" s="13" t="n">
+      <c r="F24" s="14" t="n">
         <f aca="false">E24+C24</f>
         <v>5</v>
       </c>
-      <c r="G24" s="13" t="n">
+      <c r="G24" s="14" t="n">
         <f aca="false">F24+D24</f>
         <v>5</v>
       </c>
-      <c r="H24" s="6" t="s">
+      <c r="H24" s="7" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="7" t="s">
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="8" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="8" t="s">
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="B28" s="8" t="s">
+      <c r="B28" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="H28" s="8" t="s">
+      <c r="H28" s="9" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="9" t="s">
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="B29" s="12" t="n">
+      <c r="B29" s="13" t="n">
         <v>20</v>
       </c>
-      <c r="H29" s="6" t="s">
+      <c r="H29" s="7" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="9" t="s">
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="B30" s="12" t="n">
+      <c r="B30" s="13" t="n">
         <v>0.6</v>
       </c>
-      <c r="H30" s="6" t="s">
+      <c r="H30" s="7" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="9" t="s">
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="B31" s="12" t="n">
+      <c r="B31" s="13" t="n">
         <v>3</v>
       </c>
-      <c r="H31" s="6" t="s">
+      <c r="H31" s="7" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="9" t="s">
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="B32" s="12" t="n">
+      <c r="B32" s="13" t="n">
         <v>4</v>
       </c>
-      <c r="H32" s="6" t="s">
+      <c r="H32" s="7" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="9" t="s">
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="B33" s="12" t="n">
+      <c r="B33" s="13" t="n">
         <v>2</v>
       </c>
-      <c r="H33" s="6" t="s">
+      <c r="H33" s="7" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="9" t="s">
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="B34" s="12" t="n">
+      <c r="B34" s="13" t="n">
         <v>4</v>
       </c>
-      <c r="H34" s="6" t="s">
+      <c r="H34" s="7" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="9" t="s">
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="10" t="s">
         <v>69</v>
       </c>
-      <c r="B35" s="12" t="n">
+      <c r="B35" s="13" t="n">
         <v>3</v>
       </c>
-      <c r="H35" s="6" t="s">
+      <c r="H35" s="7" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="7" t="s">
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="8" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="6" t="s">
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="7" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="11" t="s">
+    <row r="40" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="12" t="s">
         <v>73</v>
       </c>
-      <c r="B40" s="11" t="s">
+      <c r="B40" s="12" t="s">
         <v>74</v>
       </c>
-      <c r="C40" s="11" t="s">
+      <c r="C40" s="12" t="s">
         <v>75</v>
       </c>
-      <c r="D40" s="11" t="s">
+      <c r="D40" s="12" t="s">
         <v>76</v>
       </c>
-      <c r="E40" s="11" t="s">
+      <c r="E40" s="12" t="s">
         <v>77</v>
       </c>
-      <c r="F40" s="11" t="s">
+      <c r="F40" s="12" t="s">
         <v>78</v>
       </c>
-      <c r="G40" s="11" t="s">
+      <c r="G40" s="12" t="s">
         <v>79</v>
       </c>
-      <c r="H40" s="11" t="s">
+      <c r="H40" s="12" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="9" t="s">
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="10" t="s">
         <v>80</v>
       </c>
-      <c r="B41" s="14" t="n">
+      <c r="B41" s="15" t="n">
         <v>20</v>
       </c>
-      <c r="C41" s="14" t="n">
+      <c r="C41" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="D41" s="14" t="n">
+      <c r="D41" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="E41" s="14" t="n">
+      <c r="E41" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="F41" s="14" t="n">
+      <c r="F41" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="G41" s="14" t="n">
+      <c r="G41" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H41" s="6" t="s">
+      <c r="H41" s="7" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="9" t="s">
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="10" t="s">
         <v>82</v>
       </c>
-      <c r="B42" s="14" t="n">
+      <c r="B42" s="15" t="n">
         <v>35</v>
       </c>
-      <c r="C42" s="14" t="n">
+      <c r="C42" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="D42" s="14" t="n">
+      <c r="D42" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="E42" s="14" t="n">
+      <c r="E42" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="F42" s="14" t="n">
+      <c r="F42" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="G42" s="14" t="n">
+      <c r="G42" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="H42" s="6" t="s">
+      <c r="H42" s="7" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="9" t="s">
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="10" t="s">
         <v>84</v>
       </c>
-      <c r="B43" s="14" t="n">
+      <c r="B43" s="15" t="n">
         <v>50</v>
       </c>
-      <c r="C43" s="14" t="n">
+      <c r="C43" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="D43" s="14" t="n">
+      <c r="D43" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="E43" s="14" t="n">
+      <c r="E43" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="F43" s="14" t="n">
+      <c r="F43" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="G43" s="14" t="n">
+      <c r="G43" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="H43" s="6" t="s">
+      <c r="H43" s="7" t="s">
         <v>85</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="16" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="17" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="18" t="s">
+        <v>88</v>
+      </c>
+      <c r="B47" s="18" t="s">
+        <v>89</v>
+      </c>
+      <c r="C47" s="18" t="s">
+        <v>90</v>
+      </c>
+      <c r="H47" s="18" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="19" t="s">
+        <v>91</v>
+      </c>
+      <c r="B48" s="20" t="s">
+        <v>80</v>
+      </c>
+      <c r="C48" s="19" t="s">
+        <v>92</v>
+      </c>
+      <c r="H48" s="17" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="19" t="s">
+        <v>94</v>
+      </c>
+      <c r="B49" s="20" t="s">
+        <v>82</v>
+      </c>
+      <c r="C49" s="19" t="s">
+        <v>95</v>
+      </c>
+      <c r="H49" s="17" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="19" t="s">
+        <v>97</v>
+      </c>
+      <c r="B50" s="20" t="s">
+        <v>84</v>
+      </c>
+      <c r="C50" s="19" t="s">
+        <v>98</v>
+      </c>
+      <c r="H50" s="17" t="s">
+        <v>99</v>
       </c>
     </row>
   </sheetData>
@@ -1539,580 +1662,580 @@
   <dimension ref="A1:E36"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="2" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="2" style="1" width="14"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="5" t="s">
-        <v>86</v>
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="6" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="15" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="16"/>
-      <c r="B4" s="16" t="s">
-        <v>88</v>
-      </c>
-      <c r="C4" s="16" t="s">
-        <v>89</v>
-      </c>
-      <c r="D4" s="16" t="s">
-        <v>90</v>
-      </c>
-      <c r="E4" s="16" t="s">
+      <c r="A2" s="21" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="22"/>
+      <c r="B4" s="22" t="s">
         <v>91</v>
       </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="7" t="s">
+      <c r="C4" s="22" t="s">
+        <v>94</v>
+      </c>
+      <c r="D4" s="22" t="s">
+        <v>97</v>
+      </c>
+      <c r="E4" s="22" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="8" t="s">
         <v>73</v>
       </c>
-      <c r="B5" s="17" t="s">
+      <c r="B5" s="23" t="s">
         <v>80</v>
       </c>
-      <c r="C5" s="17" t="s">
+      <c r="C5" s="23" t="s">
         <v>82</v>
       </c>
-      <c r="D5" s="17" t="s">
+      <c r="D5" s="23" t="s">
         <v>84</v>
       </c>
-      <c r="E5" s="18" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="9" t="s">
+      <c r="E5" s="24" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="10" t="s">
         <v>74</v>
       </c>
-      <c r="B6" s="19" t="n">
+      <c r="B6" s="25" t="n">
         <f aca="false">INDEX(Assumptions!$B$41:$B$43,MATCH(B$5,Assumptions!$A$41:$A$43,0))</f>
         <v>20</v>
       </c>
-      <c r="C6" s="19" t="n">
+      <c r="C6" s="25" t="n">
         <f aca="false">INDEX(Assumptions!$B$41:$B$43,MATCH(C$5,Assumptions!$A$41:$A$43,0))</f>
         <v>35</v>
       </c>
-      <c r="D6" s="19" t="n">
+      <c r="D6" s="25" t="n">
         <f aca="false">INDEX(Assumptions!$B$41:$B$43,MATCH(D$5,Assumptions!$A$41:$A$43,0))</f>
         <v>50</v>
       </c>
-      <c r="E6" s="17" t="n">
+      <c r="E6" s="23" t="n">
         <v>35</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="9" t="s">
-        <v>92</v>
-      </c>
-      <c r="B7" s="19" t="n">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="10" t="s">
+        <v>103</v>
+      </c>
+      <c r="B7" s="25" t="n">
         <f aca="false">INDEX(Assumptions!$C$41:$C$43,MATCH(B$5,Assumptions!$A$41:$A$43,0))</f>
         <v>1</v>
       </c>
-      <c r="C7" s="19" t="n">
+      <c r="C7" s="25" t="n">
         <f aca="false">INDEX(Assumptions!$C$41:$C$43,MATCH(C$5,Assumptions!$A$41:$A$43,0))</f>
         <v>2</v>
       </c>
-      <c r="D7" s="19" t="n">
+      <c r="D7" s="25" t="n">
         <f aca="false">INDEX(Assumptions!$C$41:$C$43,MATCH(D$5,Assumptions!$A$41:$A$43,0))</f>
         <v>3</v>
       </c>
-      <c r="E7" s="17" t="n">
+      <c r="E7" s="23" t="n">
         <v>2</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="9" t="s">
-        <v>93</v>
-      </c>
-      <c r="B8" s="20" t="str">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="10" t="s">
+        <v>104</v>
+      </c>
+      <c r="B8" s="26" t="str">
         <f aca="false">CHOOSE(B7,"Deck mods only","Scripting","Full narrative")</f>
         <v>Deck mods only</v>
       </c>
-      <c r="C8" s="20" t="str">
+      <c r="C8" s="26" t="str">
         <f aca="false">CHOOSE(C7,"Deck mods only","Scripting","Full narrative")</f>
         <v>Scripting</v>
       </c>
-      <c r="D8" s="20" t="str">
+      <c r="D8" s="26" t="str">
         <f aca="false">CHOOSE(D7,"Deck mods only","Scripting","Full narrative")</f>
         <v>Full narrative</v>
       </c>
-      <c r="E8" s="20" t="str">
+      <c r="E8" s="26" t="str">
         <f aca="false">CHOOSE(E7,"Deck mods only","Scripting","Full narrative")</f>
         <v>Scripting</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="9" t="s">
-        <v>94</v>
-      </c>
-      <c r="B9" s="19" t="n">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="10" t="s">
+        <v>105</v>
+      </c>
+      <c r="B9" s="25" t="n">
         <f aca="false">INDEX(Assumptions!$D$41:$D$43,MATCH(B$5,Assumptions!$A$41:$A$43,0))</f>
         <v>3</v>
       </c>
-      <c r="C9" s="19" t="n">
+      <c r="C9" s="25" t="n">
         <f aca="false">INDEX(Assumptions!$D$41:$D$43,MATCH(C$5,Assumptions!$A$41:$A$43,0))</f>
         <v>4</v>
       </c>
-      <c r="D9" s="19" t="n">
+      <c r="D9" s="25" t="n">
         <f aca="false">INDEX(Assumptions!$D$41:$D$43,MATCH(D$5,Assumptions!$A$41:$A$43,0))</f>
         <v>5</v>
       </c>
-      <c r="E9" s="17" t="n">
+      <c r="E9" s="23" t="n">
         <v>4</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="9" t="s">
-        <v>95</v>
-      </c>
-      <c r="B10" s="19" t="n">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="10" t="s">
+        <v>106</v>
+      </c>
+      <c r="B10" s="25" t="n">
         <f aca="false">INDEX(Assumptions!$E$41:$E$43,MATCH(B$5,Assumptions!$A$41:$A$43,0))</f>
         <v>2</v>
       </c>
-      <c r="C10" s="19" t="n">
+      <c r="C10" s="25" t="n">
         <f aca="false">INDEX(Assumptions!$E$41:$E$43,MATCH(C$5,Assumptions!$A$41:$A$43,0))</f>
         <v>3</v>
       </c>
-      <c r="D10" s="19" t="n">
+      <c r="D10" s="25" t="n">
         <f aca="false">INDEX(Assumptions!$E$41:$E$43,MATCH(D$5,Assumptions!$A$41:$A$43,0))</f>
         <v>4</v>
       </c>
-      <c r="E10" s="17" t="n">
+      <c r="E10" s="23" t="n">
         <v>3</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="9" t="s">
-        <v>96</v>
-      </c>
-      <c r="B11" s="19" t="n">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="10" t="s">
+        <v>107</v>
+      </c>
+      <c r="B11" s="25" t="n">
         <f aca="false">INDEX(Assumptions!$F$41:$F$43,MATCH(B$5,Assumptions!$A$41:$A$43,0))</f>
         <v>1</v>
       </c>
-      <c r="C11" s="19" t="n">
+      <c r="C11" s="25" t="n">
         <f aca="false">INDEX(Assumptions!$F$41:$F$43,MATCH(C$5,Assumptions!$A$41:$A$43,0))</f>
         <v>2</v>
       </c>
-      <c r="D11" s="19" t="n">
+      <c r="D11" s="25" t="n">
         <f aca="false">INDEX(Assumptions!$F$41:$F$43,MATCH(D$5,Assumptions!$A$41:$A$43,0))</f>
         <v>3</v>
       </c>
-      <c r="E11" s="17" t="n">
+      <c r="E11" s="23" t="n">
         <v>2</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="9" t="s">
-        <v>97</v>
-      </c>
-      <c r="B12" s="19" t="n">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="10" t="s">
+        <v>108</v>
+      </c>
+      <c r="B12" s="25" t="n">
         <f aca="false">INDEX(Assumptions!$G$41:$G$43,MATCH(B$5,Assumptions!$A$41:$A$43,0))</f>
         <v>0</v>
       </c>
-      <c r="C12" s="19" t="n">
+      <c r="C12" s="25" t="n">
         <f aca="false">INDEX(Assumptions!$G$41:$G$43,MATCH(C$5,Assumptions!$A$41:$A$43,0))</f>
         <v>1</v>
       </c>
-      <c r="D12" s="19" t="n">
+      <c r="D12" s="25" t="n">
         <f aca="false">INDEX(Assumptions!$G$41:$G$43,MATCH(D$5,Assumptions!$A$41:$A$43,0))</f>
         <v>2</v>
       </c>
-      <c r="E12" s="17" t="n">
+      <c r="E12" s="23" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="21" t="s">
-        <v>98</v>
-      </c>
-      <c r="B14" s="22"/>
-      <c r="C14" s="22"/>
-      <c r="D14" s="22"/>
-      <c r="E14" s="22"/>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="9" t="s">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="27" t="s">
+        <v>109</v>
+      </c>
+      <c r="B14" s="28"/>
+      <c r="C14" s="28"/>
+      <c r="D14" s="28"/>
+      <c r="E14" s="28"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="B15" s="23" t="n">
+      <c r="B15" s="29" t="n">
         <f aca="false">INDEX(Assumptions!$E$19:$G$19,B7)+Assumptions!$B$33*B10+Assumptions!$B$35*B11</f>
         <v>11</v>
       </c>
-      <c r="C15" s="23" t="n">
+      <c r="C15" s="29" t="n">
         <f aca="false">INDEX(Assumptions!$E$19:$G$19,C7)+Assumptions!$B$33*C10+Assumptions!$B$35*C11</f>
         <v>32</v>
       </c>
-      <c r="D15" s="23" t="n">
+      <c r="D15" s="29" t="n">
         <f aca="false">INDEX(Assumptions!$E$19:$G$19,D7)+Assumptions!$B$33*D10+Assumptions!$B$35*D11</f>
         <v>65</v>
       </c>
-      <c r="E15" s="23" t="n">
+      <c r="E15" s="29" t="n">
         <f aca="false">INDEX(Assumptions!$E$19:$G$19,E7)+Assumptions!$B$33*E10+Assumptions!$B$35*E11</f>
         <v>32</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="9" t="s">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="B16" s="23" t="n">
+      <c r="B16" s="29" t="n">
         <f aca="false">INDEX(Assumptions!$E$20:$G$20,B7)+Assumptions!$B$31*B9</f>
         <v>9</v>
       </c>
-      <c r="C16" s="23" t="n">
+      <c r="C16" s="29" t="n">
         <f aca="false">INDEX(Assumptions!$E$20:$G$20,C7)+Assumptions!$B$31*C9</f>
         <v>20</v>
       </c>
-      <c r="D16" s="23" t="n">
+      <c r="D16" s="29" t="n">
         <f aca="false">INDEX(Assumptions!$E$20:$G$20,D7)+Assumptions!$B$31*D9</f>
         <v>37</v>
       </c>
-      <c r="E16" s="23" t="n">
+      <c r="E16" s="29" t="n">
         <f aca="false">INDEX(Assumptions!$E$20:$G$20,E7)+Assumptions!$B$31*E9</f>
         <v>20</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="9" t="s">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="B17" s="23" t="n">
+      <c r="B17" s="29" t="n">
         <f aca="false">INDEX(Assumptions!$E$21:$G$21,B7)+Assumptions!$B$30*MAX(0,B6-Assumptions!$B$29)+Assumptions!$B$32*B10</f>
         <v>28</v>
       </c>
-      <c r="C17" s="23" t="n">
+      <c r="C17" s="29" t="n">
         <f aca="false">INDEX(Assumptions!$E$21:$G$21,C7)+Assumptions!$B$30*MAX(0,C6-Assumptions!$B$29)+Assumptions!$B$32*C10</f>
         <v>41</v>
       </c>
-      <c r="D17" s="23" t="n">
+      <c r="D17" s="29" t="n">
         <f aca="false">INDEX(Assumptions!$E$21:$G$21,D7)+Assumptions!$B$30*MAX(0,D6-Assumptions!$B$29)+Assumptions!$B$32*D10</f>
         <v>54</v>
       </c>
-      <c r="E17" s="23" t="n">
+      <c r="E17" s="29" t="n">
         <f aca="false">INDEX(Assumptions!$E$21:$G$21,E7)+Assumptions!$B$30*MAX(0,E6-Assumptions!$B$29)+Assumptions!$B$32*E10</f>
         <v>41</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="9" t="s">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="B18" s="23" t="n">
+      <c r="B18" s="29" t="n">
         <f aca="false">INDEX(Assumptions!$E$22:$G$22,B7)</f>
         <v>3</v>
       </c>
-      <c r="C18" s="23" t="n">
+      <c r="C18" s="29" t="n">
         <f aca="false">INDEX(Assumptions!$E$22:$G$22,C7)</f>
         <v>3</v>
       </c>
-      <c r="D18" s="23" t="n">
+      <c r="D18" s="29" t="n">
         <f aca="false">INDEX(Assumptions!$E$22:$G$22,D7)</f>
         <v>8</v>
       </c>
-      <c r="E18" s="23" t="n">
+      <c r="E18" s="29" t="n">
         <f aca="false">INDEX(Assumptions!$E$22:$G$22,E7)</f>
         <v>3</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="9" t="s">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="B19" s="23" t="n">
+      <c r="B19" s="29" t="n">
         <f aca="false">INDEX(Assumptions!$E$23:$G$23,B7)+Assumptions!$B$34*B11</f>
         <v>10</v>
       </c>
-      <c r="C19" s="23" t="n">
+      <c r="C19" s="29" t="n">
         <f aca="false">INDEX(Assumptions!$E$23:$G$23,C7)+Assumptions!$B$34*C11</f>
         <v>14</v>
       </c>
-      <c r="D19" s="23" t="n">
+      <c r="D19" s="29" t="n">
         <f aca="false">INDEX(Assumptions!$E$23:$G$23,D7)+Assumptions!$B$34*D11</f>
         <v>18</v>
       </c>
-      <c r="E19" s="23" t="n">
+      <c r="E19" s="29" t="n">
         <f aca="false">INDEX(Assumptions!$E$23:$G$23,E7)+Assumptions!$B$34*E11</f>
         <v>14</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="9" t="s">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="B20" s="23" t="n">
+      <c r="B20" s="29" t="n">
         <f aca="false">INDEX(Assumptions!$E$24:$G$24,B7)</f>
         <v>5</v>
       </c>
-      <c r="C20" s="23" t="n">
+      <c r="C20" s="29" t="n">
         <f aca="false">INDEX(Assumptions!$E$24:$G$24,C7)</f>
         <v>5</v>
       </c>
-      <c r="D20" s="23" t="n">
+      <c r="D20" s="29" t="n">
         <f aca="false">INDEX(Assumptions!$E$24:$G$24,D7)</f>
         <v>5</v>
       </c>
-      <c r="E20" s="23" t="n">
+      <c r="E20" s="29" t="n">
         <f aca="false">INDEX(Assumptions!$E$24:$G$24,E7)</f>
         <v>5</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="7" t="s">
-        <v>99</v>
-      </c>
-      <c r="B21" s="24" t="n">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="8" t="s">
+        <v>110</v>
+      </c>
+      <c r="B21" s="30" t="n">
         <f aca="false">SUM(B15:B20)</f>
         <v>66</v>
       </c>
-      <c r="C21" s="24" t="n">
+      <c r="C21" s="30" t="n">
         <f aca="false">SUM(C15:C20)</f>
         <v>115</v>
       </c>
-      <c r="D21" s="24" t="n">
+      <c r="D21" s="30" t="n">
         <f aca="false">SUM(D15:D20)</f>
         <v>187</v>
       </c>
-      <c r="E21" s="24" t="n">
+      <c r="E21" s="30" t="n">
         <f aca="false">SUM(E15:E20)</f>
         <v>115</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="21" t="s">
-        <v>100</v>
-      </c>
-      <c r="B23" s="22"/>
-      <c r="C23" s="22"/>
-      <c r="D23" s="22"/>
-      <c r="E23" s="22"/>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="9" t="s">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="27" t="s">
+        <v>111</v>
+      </c>
+      <c r="B23" s="28"/>
+      <c r="C23" s="28"/>
+      <c r="D23" s="28"/>
+      <c r="E23" s="28"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="B24" s="25" t="n">
+      <c r="B24" s="31" t="n">
         <f aca="false">B15*Assumptions!$B$6</f>
         <v>2035</v>
       </c>
-      <c r="C24" s="25" t="n">
+      <c r="C24" s="31" t="n">
         <f aca="false">C15*Assumptions!$B$6</f>
         <v>5920</v>
       </c>
-      <c r="D24" s="25" t="n">
+      <c r="D24" s="31" t="n">
         <f aca="false">D15*Assumptions!$B$6</f>
         <v>12025</v>
       </c>
-      <c r="E24" s="25" t="n">
+      <c r="E24" s="31" t="n">
         <f aca="false">E15*Assumptions!$B$6</f>
         <v>5920</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="9" t="s">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="B25" s="25" t="n">
+      <c r="B25" s="31" t="n">
         <f aca="false">B16*Assumptions!$B$7</f>
         <v>1665</v>
       </c>
-      <c r="C25" s="25" t="n">
+      <c r="C25" s="31" t="n">
         <f aca="false">C16*Assumptions!$B$7</f>
         <v>3700</v>
       </c>
-      <c r="D25" s="25" t="n">
+      <c r="D25" s="31" t="n">
         <f aca="false">D16*Assumptions!$B$7</f>
         <v>6845</v>
       </c>
-      <c r="E25" s="25" t="n">
+      <c r="E25" s="31" t="n">
         <f aca="false">E16*Assumptions!$B$7</f>
         <v>3700</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="9" t="s">
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="B26" s="25" t="n">
+      <c r="B26" s="31" t="n">
         <f aca="false">B17*Assumptions!$B$8</f>
         <v>4900</v>
       </c>
-      <c r="C26" s="25" t="n">
+      <c r="C26" s="31" t="n">
         <f aca="false">C17*Assumptions!$B$8</f>
         <v>7175</v>
       </c>
-      <c r="D26" s="25" t="n">
+      <c r="D26" s="31" t="n">
         <f aca="false">D17*Assumptions!$B$8</f>
         <v>9450</v>
       </c>
-      <c r="E26" s="25" t="n">
+      <c r="E26" s="31" t="n">
         <f aca="false">E17*Assumptions!$B$8</f>
         <v>7175</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="9" t="s">
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="B27" s="25" t="n">
+      <c r="B27" s="31" t="n">
         <f aca="false">B18*Assumptions!$B$9</f>
         <v>600</v>
       </c>
-      <c r="C27" s="25" t="n">
+      <c r="C27" s="31" t="n">
         <f aca="false">C18*Assumptions!$B$9</f>
         <v>600</v>
       </c>
-      <c r="D27" s="25" t="n">
+      <c r="D27" s="31" t="n">
         <f aca="false">D18*Assumptions!$B$9</f>
         <v>1600</v>
       </c>
-      <c r="E27" s="25" t="n">
+      <c r="E27" s="31" t="n">
         <f aca="false">E18*Assumptions!$B$9</f>
         <v>600</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="9" t="s">
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="B28" s="25" t="n">
+      <c r="B28" s="31" t="n">
         <f aca="false">B19*Assumptions!$B$10</f>
         <v>1750</v>
       </c>
-      <c r="C28" s="25" t="n">
+      <c r="C28" s="31" t="n">
         <f aca="false">C19*Assumptions!$B$10</f>
         <v>2450</v>
       </c>
-      <c r="D28" s="25" t="n">
+      <c r="D28" s="31" t="n">
         <f aca="false">D19*Assumptions!$B$10</f>
         <v>3150</v>
       </c>
-      <c r="E28" s="25" t="n">
+      <c r="E28" s="31" t="n">
         <f aca="false">E19*Assumptions!$B$10</f>
         <v>2450</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="9" t="s">
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="B29" s="25" t="n">
+      <c r="B29" s="31" t="n">
         <f aca="false">B20*Assumptions!$B$11</f>
         <v>500</v>
       </c>
-      <c r="C29" s="25" t="n">
+      <c r="C29" s="31" t="n">
         <f aca="false">C20*Assumptions!$B$11</f>
         <v>500</v>
       </c>
-      <c r="D29" s="25" t="n">
+      <c r="D29" s="31" t="n">
         <f aca="false">D20*Assumptions!$B$11</f>
         <v>500</v>
       </c>
-      <c r="E29" s="25" t="n">
+      <c r="E29" s="31" t="n">
         <f aca="false">E20*Assumptions!$B$11</f>
         <v>500</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="7" t="s">
-        <v>101</v>
-      </c>
-      <c r="B30" s="26" t="n">
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="8" t="s">
+        <v>112</v>
+      </c>
+      <c r="B30" s="32" t="n">
         <f aca="false">SUM(B24:B29)</f>
         <v>11450</v>
       </c>
-      <c r="C30" s="26" t="n">
+      <c r="C30" s="32" t="n">
         <f aca="false">SUM(C24:C29)</f>
         <v>20345</v>
       </c>
-      <c r="D30" s="26" t="n">
+      <c r="D30" s="32" t="n">
         <f aca="false">SUM(D24:D29)</f>
         <v>33570</v>
       </c>
-      <c r="E30" s="26" t="n">
+      <c r="E30" s="32" t="n">
         <f aca="false">SUM(E24:E29)</f>
         <v>20345</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="9" t="s">
-        <v>102</v>
-      </c>
-      <c r="B31" s="25" t="n">
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="10" t="s">
+        <v>113</v>
+      </c>
+      <c r="B31" s="31" t="n">
         <f aca="false">B12*Assumptions!$B$12</f>
         <v>0</v>
       </c>
-      <c r="C31" s="25" t="n">
+      <c r="C31" s="31" t="n">
         <f aca="false">C12*Assumptions!$B$12</f>
         <v>3500</v>
       </c>
-      <c r="D31" s="25" t="n">
+      <c r="D31" s="31" t="n">
         <f aca="false">D12*Assumptions!$B$12</f>
         <v>7000</v>
       </c>
-      <c r="E31" s="25" t="n">
+      <c r="E31" s="31" t="n">
         <f aca="false">E12*Assumptions!$B$12</f>
         <v>3500</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="7" t="s">
-        <v>103</v>
-      </c>
-      <c r="B32" s="26" t="n">
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="8" t="s">
+        <v>114</v>
+      </c>
+      <c r="B32" s="32" t="n">
         <f aca="false">B30+B31</f>
         <v>11450</v>
       </c>
-      <c r="C32" s="26" t="n">
+      <c r="C32" s="32" t="n">
         <f aca="false">C30+C31</f>
         <v>23845</v>
       </c>
-      <c r="D32" s="26" t="n">
+      <c r="D32" s="32" t="n">
         <f aca="false">D30+D31</f>
         <v>40570</v>
       </c>
-      <c r="E32" s="26" t="n">
+      <c r="E32" s="32" t="n">
         <f aca="false">E30+E31</f>
         <v>23845</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="7" t="s">
-        <v>104</v>
-      </c>
-      <c r="B33" s="26" t="n">
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="8" t="s">
+        <v>115</v>
+      </c>
+      <c r="B33" s="32" t="n">
         <f aca="false">MROUND(B32,Assumptions!$B$13)</f>
         <v>11500</v>
       </c>
-      <c r="C33" s="26" t="n">
+      <c r="C33" s="32" t="n">
         <f aca="false">MROUND(C32,Assumptions!$B$13)</f>
         <v>23750</v>
       </c>
-      <c r="D33" s="26" t="n">
+      <c r="D33" s="32" t="n">
         <f aca="false">MROUND(D32,Assumptions!$B$13)</f>
         <v>40500</v>
       </c>
-      <c r="E33" s="26" t="n">
+      <c r="E33" s="32" t="n">
         <f aca="false">MROUND(E32,Assumptions!$B$13)</f>
         <v>23750</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="7" t="s">
-        <v>105</v>
-      </c>
-      <c r="B35" s="26" t="n">
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="8" t="s">
+        <v>116</v>
+      </c>
+      <c r="B35" s="32" t="n">
         <f aca="false">SUM(B33:D33)</f>
         <v>75750</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="6" t="s">
-        <v>106</v>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="7" t="s">
+        <v>117</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Simplify pricing: on-site days stepper (0 = off), absolute depth hours, round up to nearest 100
</commit_message>
<xml_diff>
--- a/pricing-model.xlsx
+++ b/pricing-model.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="115">
   <si>
     <t xml:space="preserve">AWS 1P Public Sector Symposiums - Pricing Model</t>
   </si>
@@ -51,7 +51,7 @@
     <t xml:space="preserve">THE MATH, PER DECK</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Writing depth sets cumulative base hours (each level adds onto the previous).</t>
+    <t xml:space="preserve">1. Writing depth sets absolute base hours per level.</t>
   </si>
   <si>
     <t xml:space="preserve">2. Modifiers add hours: slides above 20 add design time, each speaker adds speaker management, each edit round adds design and writing, each dry run adds PM and writing.</t>
@@ -60,7 +60,7 @@
     <t xml:space="preserve">3. Cost = sum of role hours x rates, plus flat on-site day rate x days.</t>
   </si>
   <si>
-    <t xml:space="preserve">4. Headline prices round to the nearest $250. Program total = sum of the three rounded city prices.</t>
+    <t xml:space="preserve">4. Headline prices round UP to the nearest $100. Program total = sum of the three rounded city prices.</t>
   </si>
   <si>
     <t xml:space="preserve">ALL NUMBERS ARE PLACEHOLDERS PENDING CONFIRMATION. Estimate, not a quote.</t>
@@ -69,7 +69,7 @@
     <t xml:space="preserve">Pricing Model Assumptions</t>
   </si>
   <si>
-    <t xml:space="preserve">Blue = editable input. Black = calculated. Config key shows where each value lives in pricing.config.js.</t>
+    <t xml:space="preserve">Blue = editable input. Black = calculated. Config key shows where each value lives in pricing.config.js. On-site days of 0 = no on-site support.</t>
   </si>
   <si>
     <t xml:space="preserve">Role rates</t>
@@ -135,55 +135,46 @@
     <t xml:space="preserve">onSite.dayRate</t>
   </si>
   <si>
-    <t xml:space="preserve">Round prices to nearest</t>
+    <t xml:space="preserve">Round prices UP to nearest</t>
   </si>
   <si>
     <t xml:space="preserve">$</t>
   </si>
   <si>
-    <t xml:space="preserve">roundTo</t>
+    <t xml:space="preserve">roundUpTo</t>
   </si>
   <si>
     <t xml:space="preserve">Base hours per deck by writing depth</t>
   </si>
   <si>
-    <t xml:space="preserve">Adds are cumulative, matching the config: each level starts from the previous level and adds hours.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">L1 add: Deck mods only</t>
-  </si>
-  <si>
-    <t xml:space="preserve">L2 add: Scripting from framework</t>
-  </si>
-  <si>
-    <t xml:space="preserve">L3 add: Full narrative + scripting</t>
-  </si>
-  <si>
-    <t xml:space="preserve">L1 total</t>
-  </si>
-  <si>
-    <t xml:space="preserve">L2 total</t>
-  </si>
-  <si>
-    <t xml:space="preserve">L3 total</t>
-  </si>
-  <si>
-    <t xml:space="preserve">depthLevels hours: writing</t>
-  </si>
-  <si>
-    <t xml:space="preserve">depthLevels hours: speakerMgmt</t>
-  </si>
-  <si>
-    <t xml:space="preserve">depthLevels hours: design</t>
-  </si>
-  <si>
-    <t xml:space="preserve">depthLevels hours: designDir</t>
-  </si>
-  <si>
-    <t xml:space="preserve">depthLevels hours: pm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">depthLevels hours: qc</t>
+    <t xml:space="preserve">Absolute base hours per deck for each level, matching depthLevels[].hours in the config.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L1: Deck mods only</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L2: Scripting from framework</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L3: Full narrative + scripting</t>
+  </si>
+  <si>
+    <t xml:space="preserve">depthLevels[].hours.writing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">depthLevels[].hours.speakerMgmt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">depthLevels[].hours.design</t>
+  </si>
+  <si>
+    <t xml:space="preserve">depthLevels[].hours.designDir</t>
+  </si>
+  <si>
+    <t xml:space="preserve">depthLevels[].hours.pm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">depthLevels[].hours.qc</t>
   </si>
   <si>
     <t xml:space="preserve">Modifiers (added on top of base hours)</t>
@@ -327,7 +318,7 @@
     <t xml:space="preserve">Per-Deck Pricing Calculator</t>
   </si>
   <si>
-    <t xml:space="preserve">Tiers are service levels, not locations: any symposium can run at any tier. The blue tier name per city defaults to OUR recommended starting point (based on readiness) and is fully changeable. Custom column is free-form. Estimate, not a quote.</t>
+    <t xml:space="preserve">Tiers are service levels, not locations: any symposium can run at any tier. The blue tier name per city defaults to OUR recommended starting point (based on readiness) and is fully changeable. Custom column is free-form. Headline prices round UP to the nearest \$100; the breakdown shows exact math. Estimate, not a quote.</t>
   </si>
   <si>
     <t xml:space="preserve">Custom</t>
@@ -369,7 +360,7 @@
     <t xml:space="preserve">Per-deck total (exact)</t>
   </si>
   <si>
-    <t xml:space="preserve">Per-deck total (rounded)</t>
+    <t xml:space="preserve">Per-deck total (rounded up)</t>
   </si>
   <si>
     <t xml:space="preserve">Program total (London + Ottawa + Canberra, rounded)</t>
@@ -521,15 +512,11 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="26">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -546,27 +533,27 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -574,31 +561,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -630,11 +593,11 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -909,88 +872,88 @@
   <dimension ref="A1:A18"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="110"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="110"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
+    <row r="2" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3"/>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4" t="s">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="2"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3" t="s">
+    <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3" t="s">
+    <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="3"/>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="4" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="2"/>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="3" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="3" t="s">
+    <row r="10" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="2" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="3"/>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="4" t="s">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="2"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="3" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="3" t="s">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="3" t="s">
+    <row r="14" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="2" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="3" t="s">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="2" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="3" t="s">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="2" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="3"/>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="5" t="s">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="2"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="4" t="s">
         <v>13</v>
       </c>
     </row>
@@ -1013,634 +976,556 @@
   <dimension ref="A1:H50"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="2" style="1" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="5" style="1" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="2" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="5" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="30"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="6" t="s">
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="5" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="7" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="6" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="8" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="7" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="9" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="B5" s="9" t="s">
+      <c r="B5" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="C5" s="9" t="s">
+      <c r="C5" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="H5" s="9" t="s">
+      <c r="H5" s="8" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="10" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="B6" s="11" t="n">
+      <c r="B6" s="10" t="n">
         <v>185</v>
       </c>
-      <c r="C6" s="10" t="s">
+      <c r="C6" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="H6" s="7" t="s">
+      <c r="H6" s="6" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="10" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="B7" s="11" t="n">
+      <c r="B7" s="10" t="n">
         <v>185</v>
       </c>
-      <c r="C7" s="10" t="s">
+      <c r="C7" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="H7" s="7" t="s">
+      <c r="H7" s="6" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="10" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="B8" s="11" t="n">
+      <c r="B8" s="10" t="n">
         <v>175</v>
       </c>
-      <c r="C8" s="10" t="s">
+      <c r="C8" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="H8" s="7" t="s">
+      <c r="H8" s="6" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="10" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="B9" s="11" t="n">
+      <c r="B9" s="10" t="n">
         <v>200</v>
       </c>
-      <c r="C9" s="10" t="s">
+      <c r="C9" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="H9" s="7" t="s">
+      <c r="H9" s="6" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="10" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="B10" s="11" t="n">
+      <c r="B10" s="10" t="n">
         <v>175</v>
       </c>
-      <c r="C10" s="10" t="s">
+      <c r="C10" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="H10" s="7" t="s">
+      <c r="H10" s="6" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="10" t="s">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="B11" s="11" t="n">
+      <c r="B11" s="10" t="n">
         <v>100</v>
       </c>
-      <c r="C11" s="10" t="s">
+      <c r="C11" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="H11" s="7" t="s">
+      <c r="H11" s="6" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="10" t="s">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="B12" s="11" t="n">
+      <c r="B12" s="10" t="n">
         <v>3500</v>
       </c>
-      <c r="C12" s="10" t="s">
+      <c r="C12" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="H12" s="7" t="s">
+      <c r="H12" s="6" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="10" t="s">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="B13" s="11" t="n">
-        <v>250</v>
-      </c>
-      <c r="C13" s="10" t="s">
+      <c r="B13" s="10" t="n">
+        <v>100</v>
+      </c>
+      <c r="C13" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="H13" s="7" t="s">
+      <c r="H13" s="6" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="8" t="s">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="7" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="7" t="s">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="6" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="12" t="s">
+    <row r="18" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="B18" s="12" t="s">
+      <c r="B18" s="11" t="s">
         <v>42</v>
       </c>
-      <c r="C18" s="12" t="s">
+      <c r="C18" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="D18" s="12" t="s">
+      <c r="D18" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="E18" s="12" t="s">
+      <c r="E18" s="11"/>
+      <c r="F18" s="11"/>
+      <c r="G18" s="11"/>
+      <c r="H18" s="11" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="B19" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="C19" s="12" t="n">
+        <v>20</v>
+      </c>
+      <c r="D19" s="12" t="n">
+        <v>48</v>
+      </c>
+      <c r="H19" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="F18" s="12" t="s">
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="B20" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="D20" s="12" t="n">
+        <v>22</v>
+      </c>
+      <c r="H20" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="G18" s="12" t="s">
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="B21" s="12" t="n">
+        <v>20</v>
+      </c>
+      <c r="C21" s="12" t="n">
+        <v>20</v>
+      </c>
+      <c r="D21" s="12" t="n">
+        <v>20</v>
+      </c>
+      <c r="H21" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="H18" s="12" t="s">
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="B22" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="C22" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="D22" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="H22" s="6" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="B23" s="12" t="n">
+        <v>6</v>
+      </c>
+      <c r="C23" s="12" t="n">
+        <v>6</v>
+      </c>
+      <c r="D23" s="12" t="n">
+        <v>6</v>
+      </c>
+      <c r="H23" s="6" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="B24" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="C24" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="D24" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="H24" s="6" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="7" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="B28" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="H28" s="8" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="10" t="s">
-        <v>21</v>
-      </c>
-      <c r="B19" s="13" t="n">
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="B29" s="12" t="n">
+        <v>20</v>
+      </c>
+      <c r="H29" s="6" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="B30" s="12" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="H30" s="6" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="B31" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="H31" s="6" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="9" t="s">
+        <v>60</v>
+      </c>
+      <c r="B32" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="C19" s="13" t="n">
-        <v>16</v>
-      </c>
-      <c r="D19" s="13" t="n">
-        <v>28</v>
-      </c>
-      <c r="E19" s="14" t="n">
-        <f aca="false">B19</f>
+      <c r="H32" s="6" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="9" t="s">
+        <v>62</v>
+      </c>
+      <c r="B33" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="H33" s="6" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="B34" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="F19" s="14" t="n">
-        <f aca="false">E19+C19</f>
+      <c r="H34" s="6" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="B35" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="H35" s="6" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="7" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="6" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="11" t="s">
+        <v>70</v>
+      </c>
+      <c r="B40" s="11" t="s">
+        <v>71</v>
+      </c>
+      <c r="C40" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="D40" s="11" t="s">
+        <v>73</v>
+      </c>
+      <c r="E40" s="11" t="s">
+        <v>74</v>
+      </c>
+      <c r="F40" s="11" t="s">
+        <v>75</v>
+      </c>
+      <c r="G40" s="11" t="s">
+        <v>76</v>
+      </c>
+      <c r="H40" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="G19" s="14" t="n">
-        <f aca="false">F19+D19</f>
-        <v>48</v>
-      </c>
-      <c r="H19" s="7" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="10" t="s">
-        <v>24</v>
-      </c>
-      <c r="B20" s="13" t="n">
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="B41" s="13" t="n">
+        <v>20</v>
+      </c>
+      <c r="C41" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="D41" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="E41" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="F41" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="G41" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="C20" s="13" t="n">
-        <v>8</v>
-      </c>
-      <c r="D20" s="13" t="n">
-        <v>14</v>
-      </c>
-      <c r="E20" s="14" t="n">
-        <f aca="false">B20</f>
-        <v>0</v>
-      </c>
-      <c r="F20" s="14" t="n">
-        <f aca="false">E20+C20</f>
-        <v>8</v>
-      </c>
-      <c r="G20" s="14" t="n">
-        <f aca="false">F20+D20</f>
-        <v>22</v>
-      </c>
-      <c r="H20" s="7" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="B21" s="13" t="n">
+      <c r="H41" s="6" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="B42" s="13" t="n">
+        <v>35</v>
+      </c>
+      <c r="C42" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="D42" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="E42" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="F42" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="G42" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="H42" s="6" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="B43" s="13" t="n">
+        <v>50</v>
+      </c>
+      <c r="C43" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="D43" s="13" t="n">
+        <v>5</v>
+      </c>
+      <c r="E43" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="F43" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="G43" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="H43" s="6" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="7" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="6" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="B47" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="C47" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="H47" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="C21" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="D21" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="E21" s="14" t="n">
-        <f aca="false">B21</f>
-        <v>20</v>
-      </c>
-      <c r="F21" s="14" t="n">
-        <f aca="false">E21+C21</f>
-        <v>20</v>
-      </c>
-      <c r="G21" s="14" t="n">
-        <f aca="false">F21+D21</f>
-        <v>20</v>
-      </c>
-      <c r="H21" s="7" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="10" t="s">
-        <v>28</v>
-      </c>
-      <c r="B22" s="13" t="n">
-        <v>3</v>
-      </c>
-      <c r="C22" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="D22" s="13" t="n">
-        <v>5</v>
-      </c>
-      <c r="E22" s="14" t="n">
-        <f aca="false">B22</f>
-        <v>3</v>
-      </c>
-      <c r="F22" s="14" t="n">
-        <f aca="false">E22+C22</f>
-        <v>3</v>
-      </c>
-      <c r="G22" s="14" t="n">
-        <f aca="false">F22+D22</f>
-        <v>8</v>
-      </c>
-      <c r="H22" s="7" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="B23" s="13" t="n">
-        <v>6</v>
-      </c>
-      <c r="C23" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="D23" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="E23" s="14" t="n">
-        <f aca="false">B23</f>
-        <v>6</v>
-      </c>
-      <c r="F23" s="14" t="n">
-        <f aca="false">E23+C23</f>
-        <v>6</v>
-      </c>
-      <c r="G23" s="14" t="n">
-        <f aca="false">F23+D23</f>
-        <v>6</v>
-      </c>
-      <c r="H23" s="7" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="10" t="s">
-        <v>32</v>
-      </c>
-      <c r="B24" s="13" t="n">
-        <v>5</v>
-      </c>
-      <c r="C24" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="D24" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="E24" s="14" t="n">
-        <f aca="false">B24</f>
-        <v>5</v>
-      </c>
-      <c r="F24" s="14" t="n">
-        <f aca="false">E24+C24</f>
-        <v>5</v>
-      </c>
-      <c r="G24" s="14" t="n">
-        <f aca="false">F24+D24</f>
-        <v>5</v>
-      </c>
-      <c r="H24" s="7" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="8" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="9" t="s">
-        <v>55</v>
-      </c>
-      <c r="B28" s="9" t="s">
-        <v>56</v>
-      </c>
-      <c r="H28" s="9" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="10" t="s">
-        <v>57</v>
-      </c>
-      <c r="B29" s="13" t="n">
-        <v>20</v>
-      </c>
-      <c r="H29" s="7" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="10" t="s">
-        <v>59</v>
-      </c>
-      <c r="B30" s="13" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="H30" s="7" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="10" t="s">
-        <v>61</v>
-      </c>
-      <c r="B31" s="13" t="n">
-        <v>3</v>
-      </c>
-      <c r="H31" s="7" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="10" t="s">
-        <v>63</v>
-      </c>
-      <c r="B32" s="13" t="n">
-        <v>4</v>
-      </c>
-      <c r="H32" s="7" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="10" t="s">
-        <v>65</v>
-      </c>
-      <c r="B33" s="13" t="n">
-        <v>2</v>
-      </c>
-      <c r="H33" s="7" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="10" t="s">
-        <v>67</v>
-      </c>
-      <c r="B34" s="13" t="n">
-        <v>4</v>
-      </c>
-      <c r="H34" s="7" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="10" t="s">
-        <v>69</v>
-      </c>
-      <c r="B35" s="13" t="n">
-        <v>3</v>
-      </c>
-      <c r="H35" s="7" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="8" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="7" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="40" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="12" t="s">
-        <v>73</v>
-      </c>
-      <c r="B40" s="12" t="s">
-        <v>74</v>
-      </c>
-      <c r="C40" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="D40" s="12" t="s">
-        <v>76</v>
-      </c>
-      <c r="E40" s="12" t="s">
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="B48" s="13" t="s">
         <v>77</v>
       </c>
-      <c r="F40" s="12" t="s">
-        <v>78</v>
-      </c>
-      <c r="G40" s="12" t="s">
+      <c r="C48" s="9" t="s">
+        <v>89</v>
+      </c>
+      <c r="H48" s="6" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="B49" s="13" t="s">
         <v>79</v>
       </c>
-      <c r="H40" s="12" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A41" s="10" t="s">
-        <v>80</v>
-      </c>
-      <c r="B41" s="15" t="n">
-        <v>20</v>
-      </c>
-      <c r="C41" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="D41" s="15" t="n">
-        <v>3</v>
-      </c>
-      <c r="E41" s="15" t="n">
-        <v>2</v>
-      </c>
-      <c r="F41" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="G41" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H41" s="7" t="s">
+      <c r="C49" s="9" t="s">
+        <v>92</v>
+      </c>
+      <c r="H49" s="6" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="B50" s="13" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="10" t="s">
-        <v>82</v>
-      </c>
-      <c r="B42" s="15" t="n">
-        <v>35</v>
-      </c>
-      <c r="C42" s="15" t="n">
-        <v>2</v>
-      </c>
-      <c r="D42" s="15" t="n">
-        <v>4</v>
-      </c>
-      <c r="E42" s="15" t="n">
-        <v>3</v>
-      </c>
-      <c r="F42" s="15" t="n">
-        <v>2</v>
-      </c>
-      <c r="G42" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="H42" s="7" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A43" s="10" t="s">
-        <v>84</v>
-      </c>
-      <c r="B43" s="15" t="n">
-        <v>50</v>
-      </c>
-      <c r="C43" s="15" t="n">
-        <v>3</v>
-      </c>
-      <c r="D43" s="15" t="n">
-        <v>5</v>
-      </c>
-      <c r="E43" s="15" t="n">
-        <v>4</v>
-      </c>
-      <c r="F43" s="15" t="n">
-        <v>3</v>
-      </c>
-      <c r="G43" s="15" t="n">
-        <v>2</v>
-      </c>
-      <c r="H43" s="7" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="16" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="17" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="18" t="s">
-        <v>88</v>
-      </c>
-      <c r="B47" s="18" t="s">
-        <v>89</v>
-      </c>
-      <c r="C47" s="18" t="s">
-        <v>90</v>
-      </c>
-      <c r="H47" s="18" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="19" t="s">
-        <v>91</v>
-      </c>
-      <c r="B48" s="20" t="s">
-        <v>80</v>
-      </c>
-      <c r="C48" s="19" t="s">
-        <v>92</v>
-      </c>
-      <c r="H48" s="17" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="19" t="s">
-        <v>94</v>
-      </c>
-      <c r="B49" s="20" t="s">
-        <v>82</v>
-      </c>
-      <c r="C49" s="19" t="s">
+      <c r="C50" s="9" t="s">
         <v>95</v>
       </c>
-      <c r="H49" s="17" t="s">
+      <c r="H50" s="6" t="s">
         <v>96</v>
-      </c>
-    </row>
-    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="19" t="s">
-        <v>97</v>
-      </c>
-      <c r="B50" s="20" t="s">
-        <v>84</v>
-      </c>
-      <c r="C50" s="19" t="s">
-        <v>98</v>
-      </c>
-      <c r="H50" s="17" t="s">
-        <v>99</v>
       </c>
     </row>
   </sheetData>
@@ -1662,580 +1547,580 @@
   <dimension ref="A1:E36"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="2" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="2" style="0" width="14"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="6" t="s">
-        <v>100</v>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="5" t="s">
+        <v>97</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="21" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="22"/>
-      <c r="B4" s="22" t="s">
+      <c r="A2" s="14" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="15"/>
+      <c r="B4" s="15" t="s">
+        <v>88</v>
+      </c>
+      <c r="C4" s="15" t="s">
         <v>91</v>
       </c>
-      <c r="C4" s="22" t="s">
+      <c r="D4" s="15" t="s">
         <v>94</v>
       </c>
-      <c r="D4" s="22" t="s">
-        <v>97</v>
-      </c>
-      <c r="E4" s="22" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="8" t="s">
-        <v>73</v>
-      </c>
-      <c r="B5" s="23" t="s">
-        <v>80</v>
-      </c>
-      <c r="C5" s="23" t="s">
-        <v>82</v>
-      </c>
-      <c r="D5" s="23" t="s">
-        <v>84</v>
-      </c>
-      <c r="E5" s="24" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="10" t="s">
-        <v>74</v>
-      </c>
-      <c r="B6" s="25" t="n">
+      <c r="E4" s="15" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="B5" s="16" t="s">
+        <v>77</v>
+      </c>
+      <c r="C5" s="16" t="s">
+        <v>79</v>
+      </c>
+      <c r="D5" s="16" t="s">
+        <v>81</v>
+      </c>
+      <c r="E5" s="17" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="B6" s="18" t="n">
         <f aca="false">INDEX(Assumptions!$B$41:$B$43,MATCH(B$5,Assumptions!$A$41:$A$43,0))</f>
         <v>20</v>
       </c>
-      <c r="C6" s="25" t="n">
+      <c r="C6" s="18" t="n">
         <f aca="false">INDEX(Assumptions!$B$41:$B$43,MATCH(C$5,Assumptions!$A$41:$A$43,0))</f>
         <v>35</v>
       </c>
-      <c r="D6" s="25" t="n">
+      <c r="D6" s="18" t="n">
         <f aca="false">INDEX(Assumptions!$B$41:$B$43,MATCH(D$5,Assumptions!$A$41:$A$43,0))</f>
         <v>50</v>
       </c>
-      <c r="E6" s="23" t="n">
+      <c r="E6" s="16" t="n">
         <v>35</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="10" t="s">
-        <v>103</v>
-      </c>
-      <c r="B7" s="25" t="n">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="9" t="s">
+        <v>100</v>
+      </c>
+      <c r="B7" s="18" t="n">
         <f aca="false">INDEX(Assumptions!$C$41:$C$43,MATCH(B$5,Assumptions!$A$41:$A$43,0))</f>
         <v>1</v>
       </c>
-      <c r="C7" s="25" t="n">
+      <c r="C7" s="18" t="n">
         <f aca="false">INDEX(Assumptions!$C$41:$C$43,MATCH(C$5,Assumptions!$A$41:$A$43,0))</f>
         <v>2</v>
       </c>
-      <c r="D7" s="25" t="n">
+      <c r="D7" s="18" t="n">
         <f aca="false">INDEX(Assumptions!$C$41:$C$43,MATCH(D$5,Assumptions!$A$41:$A$43,0))</f>
         <v>3</v>
       </c>
-      <c r="E7" s="23" t="n">
+      <c r="E7" s="16" t="n">
         <v>2</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="10" t="s">
-        <v>104</v>
-      </c>
-      <c r="B8" s="26" t="str">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="9" t="s">
+        <v>101</v>
+      </c>
+      <c r="B8" s="19" t="str">
         <f aca="false">CHOOSE(B7,"Deck mods only","Scripting","Full narrative")</f>
         <v>Deck mods only</v>
       </c>
-      <c r="C8" s="26" t="str">
+      <c r="C8" s="19" t="str">
         <f aca="false">CHOOSE(C7,"Deck mods only","Scripting","Full narrative")</f>
         <v>Scripting</v>
       </c>
-      <c r="D8" s="26" t="str">
+      <c r="D8" s="19" t="str">
         <f aca="false">CHOOSE(D7,"Deck mods only","Scripting","Full narrative")</f>
         <v>Full narrative</v>
       </c>
-      <c r="E8" s="26" t="str">
+      <c r="E8" s="19" t="str">
         <f aca="false">CHOOSE(E7,"Deck mods only","Scripting","Full narrative")</f>
         <v>Scripting</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="10" t="s">
-        <v>105</v>
-      </c>
-      <c r="B9" s="25" t="n">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="9" t="s">
+        <v>102</v>
+      </c>
+      <c r="B9" s="18" t="n">
         <f aca="false">INDEX(Assumptions!$D$41:$D$43,MATCH(B$5,Assumptions!$A$41:$A$43,0))</f>
         <v>3</v>
       </c>
-      <c r="C9" s="25" t="n">
+      <c r="C9" s="18" t="n">
         <f aca="false">INDEX(Assumptions!$D$41:$D$43,MATCH(C$5,Assumptions!$A$41:$A$43,0))</f>
         <v>4</v>
       </c>
-      <c r="D9" s="25" t="n">
+      <c r="D9" s="18" t="n">
         <f aca="false">INDEX(Assumptions!$D$41:$D$43,MATCH(D$5,Assumptions!$A$41:$A$43,0))</f>
         <v>5</v>
       </c>
-      <c r="E9" s="23" t="n">
+      <c r="E9" s="16" t="n">
         <v>4</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="10" t="s">
-        <v>106</v>
-      </c>
-      <c r="B10" s="25" t="n">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="9" t="s">
+        <v>103</v>
+      </c>
+      <c r="B10" s="18" t="n">
         <f aca="false">INDEX(Assumptions!$E$41:$E$43,MATCH(B$5,Assumptions!$A$41:$A$43,0))</f>
         <v>2</v>
       </c>
-      <c r="C10" s="25" t="n">
+      <c r="C10" s="18" t="n">
         <f aca="false">INDEX(Assumptions!$E$41:$E$43,MATCH(C$5,Assumptions!$A$41:$A$43,0))</f>
         <v>3</v>
       </c>
-      <c r="D10" s="25" t="n">
+      <c r="D10" s="18" t="n">
         <f aca="false">INDEX(Assumptions!$E$41:$E$43,MATCH(D$5,Assumptions!$A$41:$A$43,0))</f>
         <v>4</v>
       </c>
-      <c r="E10" s="23" t="n">
+      <c r="E10" s="16" t="n">
         <v>3</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="10" t="s">
-        <v>107</v>
-      </c>
-      <c r="B11" s="25" t="n">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="B11" s="18" t="n">
         <f aca="false">INDEX(Assumptions!$F$41:$F$43,MATCH(B$5,Assumptions!$A$41:$A$43,0))</f>
         <v>1</v>
       </c>
-      <c r="C11" s="25" t="n">
+      <c r="C11" s="18" t="n">
         <f aca="false">INDEX(Assumptions!$F$41:$F$43,MATCH(C$5,Assumptions!$A$41:$A$43,0))</f>
         <v>2</v>
       </c>
-      <c r="D11" s="25" t="n">
+      <c r="D11" s="18" t="n">
         <f aca="false">INDEX(Assumptions!$F$41:$F$43,MATCH(D$5,Assumptions!$A$41:$A$43,0))</f>
         <v>3</v>
       </c>
-      <c r="E11" s="23" t="n">
+      <c r="E11" s="16" t="n">
         <v>2</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="10" t="s">
-        <v>108</v>
-      </c>
-      <c r="B12" s="25" t="n">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="9" t="s">
+        <v>105</v>
+      </c>
+      <c r="B12" s="18" t="n">
         <f aca="false">INDEX(Assumptions!$G$41:$G$43,MATCH(B$5,Assumptions!$A$41:$A$43,0))</f>
         <v>0</v>
       </c>
-      <c r="C12" s="25" t="n">
+      <c r="C12" s="18" t="n">
         <f aca="false">INDEX(Assumptions!$G$41:$G$43,MATCH(C$5,Assumptions!$A$41:$A$43,0))</f>
         <v>1</v>
       </c>
-      <c r="D12" s="25" t="n">
+      <c r="D12" s="18" t="n">
         <f aca="false">INDEX(Assumptions!$G$41:$G$43,MATCH(D$5,Assumptions!$A$41:$A$43,0))</f>
         <v>2</v>
       </c>
-      <c r="E12" s="23" t="n">
+      <c r="E12" s="16" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="27" t="s">
-        <v>109</v>
-      </c>
-      <c r="B14" s="28"/>
-      <c r="C14" s="28"/>
-      <c r="D14" s="28"/>
-      <c r="E14" s="28"/>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="10" t="s">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="20" t="s">
+        <v>106</v>
+      </c>
+      <c r="B14" s="21"/>
+      <c r="C14" s="21"/>
+      <c r="D14" s="21"/>
+      <c r="E14" s="21"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="B15" s="29" t="n">
-        <f aca="false">INDEX(Assumptions!$E$19:$G$19,B7)+Assumptions!$B$33*B10+Assumptions!$B$35*B11</f>
+      <c r="B15" s="22" t="n">
+        <f aca="false">INDEX(Assumptions!$B$19:$D$19,B7)+Assumptions!$B$33*B10+Assumptions!$B$35*B11</f>
         <v>11</v>
       </c>
-      <c r="C15" s="29" t="n">
-        <f aca="false">INDEX(Assumptions!$E$19:$G$19,C7)+Assumptions!$B$33*C10+Assumptions!$B$35*C11</f>
+      <c r="C15" s="22" t="n">
+        <f aca="false">INDEX(Assumptions!$B$19:$D$19,C7)+Assumptions!$B$33*C10+Assumptions!$B$35*C11</f>
         <v>32</v>
       </c>
-      <c r="D15" s="29" t="n">
-        <f aca="false">INDEX(Assumptions!$E$19:$G$19,D7)+Assumptions!$B$33*D10+Assumptions!$B$35*D11</f>
+      <c r="D15" s="22" t="n">
+        <f aca="false">INDEX(Assumptions!$B$19:$D$19,D7)+Assumptions!$B$33*D10+Assumptions!$B$35*D11</f>
         <v>65</v>
       </c>
-      <c r="E15" s="29" t="n">
-        <f aca="false">INDEX(Assumptions!$E$19:$G$19,E7)+Assumptions!$B$33*E10+Assumptions!$B$35*E11</f>
+      <c r="E15" s="22" t="n">
+        <f aca="false">INDEX(Assumptions!$B$19:$D$19,E7)+Assumptions!$B$33*E10+Assumptions!$B$35*E11</f>
         <v>32</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="10" t="s">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="B16" s="29" t="n">
-        <f aca="false">INDEX(Assumptions!$E$20:$G$20,B7)+Assumptions!$B$31*B9</f>
+      <c r="B16" s="22" t="n">
+        <f aca="false">INDEX(Assumptions!$B$20:$D$20,B7)+Assumptions!$B$31*B9</f>
         <v>9</v>
       </c>
-      <c r="C16" s="29" t="n">
-        <f aca="false">INDEX(Assumptions!$E$20:$G$20,C7)+Assumptions!$B$31*C9</f>
+      <c r="C16" s="22" t="n">
+        <f aca="false">INDEX(Assumptions!$B$20:$D$20,C7)+Assumptions!$B$31*C9</f>
         <v>20</v>
       </c>
-      <c r="D16" s="29" t="n">
-        <f aca="false">INDEX(Assumptions!$E$20:$G$20,D7)+Assumptions!$B$31*D9</f>
+      <c r="D16" s="22" t="n">
+        <f aca="false">INDEX(Assumptions!$B$20:$D$20,D7)+Assumptions!$B$31*D9</f>
         <v>37</v>
       </c>
-      <c r="E16" s="29" t="n">
-        <f aca="false">INDEX(Assumptions!$E$20:$G$20,E7)+Assumptions!$B$31*E9</f>
+      <c r="E16" s="22" t="n">
+        <f aca="false">INDEX(Assumptions!$B$20:$D$20,E7)+Assumptions!$B$31*E9</f>
         <v>20</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="10" t="s">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="B17" s="29" t="n">
-        <f aca="false">INDEX(Assumptions!$E$21:$G$21,B7)+Assumptions!$B$30*MAX(0,B6-Assumptions!$B$29)+Assumptions!$B$32*B10</f>
+      <c r="B17" s="22" t="n">
+        <f aca="false">INDEX(Assumptions!$B$21:$D$21,B7)+Assumptions!$B$30*MAX(0,B6-Assumptions!$B$29)+Assumptions!$B$32*B10</f>
         <v>28</v>
       </c>
-      <c r="C17" s="29" t="n">
-        <f aca="false">INDEX(Assumptions!$E$21:$G$21,C7)+Assumptions!$B$30*MAX(0,C6-Assumptions!$B$29)+Assumptions!$B$32*C10</f>
+      <c r="C17" s="22" t="n">
+        <f aca="false">INDEX(Assumptions!$B$21:$D$21,C7)+Assumptions!$B$30*MAX(0,C6-Assumptions!$B$29)+Assumptions!$B$32*C10</f>
         <v>41</v>
       </c>
-      <c r="D17" s="29" t="n">
-        <f aca="false">INDEX(Assumptions!$E$21:$G$21,D7)+Assumptions!$B$30*MAX(0,D6-Assumptions!$B$29)+Assumptions!$B$32*D10</f>
+      <c r="D17" s="22" t="n">
+        <f aca="false">INDEX(Assumptions!$B$21:$D$21,D7)+Assumptions!$B$30*MAX(0,D6-Assumptions!$B$29)+Assumptions!$B$32*D10</f>
         <v>54</v>
       </c>
-      <c r="E17" s="29" t="n">
-        <f aca="false">INDEX(Assumptions!$E$21:$G$21,E7)+Assumptions!$B$30*MAX(0,E6-Assumptions!$B$29)+Assumptions!$B$32*E10</f>
+      <c r="E17" s="22" t="n">
+        <f aca="false">INDEX(Assumptions!$B$21:$D$21,E7)+Assumptions!$B$30*MAX(0,E6-Assumptions!$B$29)+Assumptions!$B$32*E10</f>
         <v>41</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="10" t="s">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="B18" s="29" t="n">
-        <f aca="false">INDEX(Assumptions!$E$22:$G$22,B7)</f>
+      <c r="B18" s="22" t="n">
+        <f aca="false">INDEX(Assumptions!$B$22:$D$22,B7)</f>
         <v>3</v>
       </c>
-      <c r="C18" s="29" t="n">
-        <f aca="false">INDEX(Assumptions!$E$22:$G$22,C7)</f>
+      <c r="C18" s="22" t="n">
+        <f aca="false">INDEX(Assumptions!$B$22:$D$22,C7)</f>
         <v>3</v>
       </c>
-      <c r="D18" s="29" t="n">
-        <f aca="false">INDEX(Assumptions!$E$22:$G$22,D7)</f>
+      <c r="D18" s="22" t="n">
+        <f aca="false">INDEX(Assumptions!$B$22:$D$22,D7)</f>
         <v>8</v>
       </c>
-      <c r="E18" s="29" t="n">
-        <f aca="false">INDEX(Assumptions!$E$22:$G$22,E7)</f>
+      <c r="E18" s="22" t="n">
+        <f aca="false">INDEX(Assumptions!$B$22:$D$22,E7)</f>
         <v>3</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="10" t="s">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="B19" s="29" t="n">
-        <f aca="false">INDEX(Assumptions!$E$23:$G$23,B7)+Assumptions!$B$34*B11</f>
+      <c r="B19" s="22" t="n">
+        <f aca="false">INDEX(Assumptions!$B$23:$D$23,B7)+Assumptions!$B$34*B11</f>
         <v>10</v>
       </c>
-      <c r="C19" s="29" t="n">
-        <f aca="false">INDEX(Assumptions!$E$23:$G$23,C7)+Assumptions!$B$34*C11</f>
+      <c r="C19" s="22" t="n">
+        <f aca="false">INDEX(Assumptions!$B$23:$D$23,C7)+Assumptions!$B$34*C11</f>
         <v>14</v>
       </c>
-      <c r="D19" s="29" t="n">
-        <f aca="false">INDEX(Assumptions!$E$23:$G$23,D7)+Assumptions!$B$34*D11</f>
+      <c r="D19" s="22" t="n">
+        <f aca="false">INDEX(Assumptions!$B$23:$D$23,D7)+Assumptions!$B$34*D11</f>
         <v>18</v>
       </c>
-      <c r="E19" s="29" t="n">
-        <f aca="false">INDEX(Assumptions!$E$23:$G$23,E7)+Assumptions!$B$34*E11</f>
+      <c r="E19" s="22" t="n">
+        <f aca="false">INDEX(Assumptions!$B$23:$D$23,E7)+Assumptions!$B$34*E11</f>
         <v>14</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="10" t="s">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="B20" s="29" t="n">
-        <f aca="false">INDEX(Assumptions!$E$24:$G$24,B7)</f>
+      <c r="B20" s="22" t="n">
+        <f aca="false">INDEX(Assumptions!$B$24:$D$24,B7)</f>
         <v>5</v>
       </c>
-      <c r="C20" s="29" t="n">
-        <f aca="false">INDEX(Assumptions!$E$24:$G$24,C7)</f>
+      <c r="C20" s="22" t="n">
+        <f aca="false">INDEX(Assumptions!$B$24:$D$24,C7)</f>
         <v>5</v>
       </c>
-      <c r="D20" s="29" t="n">
-        <f aca="false">INDEX(Assumptions!$E$24:$G$24,D7)</f>
+      <c r="D20" s="22" t="n">
+        <f aca="false">INDEX(Assumptions!$B$24:$D$24,D7)</f>
         <v>5</v>
       </c>
-      <c r="E20" s="29" t="n">
-        <f aca="false">INDEX(Assumptions!$E$24:$G$24,E7)</f>
+      <c r="E20" s="22" t="n">
+        <f aca="false">INDEX(Assumptions!$B$24:$D$24,E7)</f>
         <v>5</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="8" t="s">
-        <v>110</v>
-      </c>
-      <c r="B21" s="30" t="n">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="7" t="s">
+        <v>107</v>
+      </c>
+      <c r="B21" s="23" t="n">
         <f aca="false">SUM(B15:B20)</f>
         <v>66</v>
       </c>
-      <c r="C21" s="30" t="n">
+      <c r="C21" s="23" t="n">
         <f aca="false">SUM(C15:C20)</f>
         <v>115</v>
       </c>
-      <c r="D21" s="30" t="n">
+      <c r="D21" s="23" t="n">
         <f aca="false">SUM(D15:D20)</f>
         <v>187</v>
       </c>
-      <c r="E21" s="30" t="n">
+      <c r="E21" s="23" t="n">
         <f aca="false">SUM(E15:E20)</f>
         <v>115</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="27" t="s">
-        <v>111</v>
-      </c>
-      <c r="B23" s="28"/>
-      <c r="C23" s="28"/>
-      <c r="D23" s="28"/>
-      <c r="E23" s="28"/>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="10" t="s">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="20" t="s">
+        <v>108</v>
+      </c>
+      <c r="B23" s="21"/>
+      <c r="C23" s="21"/>
+      <c r="D23" s="21"/>
+      <c r="E23" s="21"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="B24" s="31" t="n">
+      <c r="B24" s="24" t="n">
         <f aca="false">B15*Assumptions!$B$6</f>
         <v>2035</v>
       </c>
-      <c r="C24" s="31" t="n">
+      <c r="C24" s="24" t="n">
         <f aca="false">C15*Assumptions!$B$6</f>
         <v>5920</v>
       </c>
-      <c r="D24" s="31" t="n">
+      <c r="D24" s="24" t="n">
         <f aca="false">D15*Assumptions!$B$6</f>
         <v>12025</v>
       </c>
-      <c r="E24" s="31" t="n">
+      <c r="E24" s="24" t="n">
         <f aca="false">E15*Assumptions!$B$6</f>
         <v>5920</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="10" t="s">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="B25" s="31" t="n">
+      <c r="B25" s="24" t="n">
         <f aca="false">B16*Assumptions!$B$7</f>
         <v>1665</v>
       </c>
-      <c r="C25" s="31" t="n">
+      <c r="C25" s="24" t="n">
         <f aca="false">C16*Assumptions!$B$7</f>
         <v>3700</v>
       </c>
-      <c r="D25" s="31" t="n">
+      <c r="D25" s="24" t="n">
         <f aca="false">D16*Assumptions!$B$7</f>
         <v>6845</v>
       </c>
-      <c r="E25" s="31" t="n">
+      <c r="E25" s="24" t="n">
         <f aca="false">E16*Assumptions!$B$7</f>
         <v>3700</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="10" t="s">
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="B26" s="31" t="n">
+      <c r="B26" s="24" t="n">
         <f aca="false">B17*Assumptions!$B$8</f>
         <v>4900</v>
       </c>
-      <c r="C26" s="31" t="n">
+      <c r="C26" s="24" t="n">
         <f aca="false">C17*Assumptions!$B$8</f>
         <v>7175</v>
       </c>
-      <c r="D26" s="31" t="n">
+      <c r="D26" s="24" t="n">
         <f aca="false">D17*Assumptions!$B$8</f>
         <v>9450</v>
       </c>
-      <c r="E26" s="31" t="n">
+      <c r="E26" s="24" t="n">
         <f aca="false">E17*Assumptions!$B$8</f>
         <v>7175</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="10" t="s">
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="B27" s="31" t="n">
+      <c r="B27" s="24" t="n">
         <f aca="false">B18*Assumptions!$B$9</f>
         <v>600</v>
       </c>
-      <c r="C27" s="31" t="n">
+      <c r="C27" s="24" t="n">
         <f aca="false">C18*Assumptions!$B$9</f>
         <v>600</v>
       </c>
-      <c r="D27" s="31" t="n">
+      <c r="D27" s="24" t="n">
         <f aca="false">D18*Assumptions!$B$9</f>
         <v>1600</v>
       </c>
-      <c r="E27" s="31" t="n">
+      <c r="E27" s="24" t="n">
         <f aca="false">E18*Assumptions!$B$9</f>
         <v>600</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="10" t="s">
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="B28" s="31" t="n">
+      <c r="B28" s="24" t="n">
         <f aca="false">B19*Assumptions!$B$10</f>
         <v>1750</v>
       </c>
-      <c r="C28" s="31" t="n">
+      <c r="C28" s="24" t="n">
         <f aca="false">C19*Assumptions!$B$10</f>
         <v>2450</v>
       </c>
-      <c r="D28" s="31" t="n">
+      <c r="D28" s="24" t="n">
         <f aca="false">D19*Assumptions!$B$10</f>
         <v>3150</v>
       </c>
-      <c r="E28" s="31" t="n">
+      <c r="E28" s="24" t="n">
         <f aca="false">E19*Assumptions!$B$10</f>
         <v>2450</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="10" t="s">
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="B29" s="31" t="n">
+      <c r="B29" s="24" t="n">
         <f aca="false">B20*Assumptions!$B$11</f>
         <v>500</v>
       </c>
-      <c r="C29" s="31" t="n">
+      <c r="C29" s="24" t="n">
         <f aca="false">C20*Assumptions!$B$11</f>
         <v>500</v>
       </c>
-      <c r="D29" s="31" t="n">
+      <c r="D29" s="24" t="n">
         <f aca="false">D20*Assumptions!$B$11</f>
         <v>500</v>
       </c>
-      <c r="E29" s="31" t="n">
+      <c r="E29" s="24" t="n">
         <f aca="false">E20*Assumptions!$B$11</f>
         <v>500</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="8" t="s">
-        <v>112</v>
-      </c>
-      <c r="B30" s="32" t="n">
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="B30" s="25" t="n">
         <f aca="false">SUM(B24:B29)</f>
         <v>11450</v>
       </c>
-      <c r="C30" s="32" t="n">
+      <c r="C30" s="25" t="n">
         <f aca="false">SUM(C24:C29)</f>
         <v>20345</v>
       </c>
-      <c r="D30" s="32" t="n">
+      <c r="D30" s="25" t="n">
         <f aca="false">SUM(D24:D29)</f>
         <v>33570</v>
       </c>
-      <c r="E30" s="32" t="n">
+      <c r="E30" s="25" t="n">
         <f aca="false">SUM(E24:E29)</f>
         <v>20345</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="10" t="s">
-        <v>113</v>
-      </c>
-      <c r="B31" s="31" t="n">
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="B31" s="24" t="n">
         <f aca="false">B12*Assumptions!$B$12</f>
         <v>0</v>
       </c>
-      <c r="C31" s="31" t="n">
+      <c r="C31" s="24" t="n">
         <f aca="false">C12*Assumptions!$B$12</f>
         <v>3500</v>
       </c>
-      <c r="D31" s="31" t="n">
+      <c r="D31" s="24" t="n">
         <f aca="false">D12*Assumptions!$B$12</f>
         <v>7000</v>
       </c>
-      <c r="E31" s="31" t="n">
+      <c r="E31" s="24" t="n">
         <f aca="false">E12*Assumptions!$B$12</f>
         <v>3500</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="8" t="s">
-        <v>114</v>
-      </c>
-      <c r="B32" s="32" t="n">
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="7" t="s">
+        <v>111</v>
+      </c>
+      <c r="B32" s="25" t="n">
         <f aca="false">B30+B31</f>
         <v>11450</v>
       </c>
-      <c r="C32" s="32" t="n">
+      <c r="C32" s="25" t="n">
         <f aca="false">C30+C31</f>
         <v>23845</v>
       </c>
-      <c r="D32" s="32" t="n">
+      <c r="D32" s="25" t="n">
         <f aca="false">D30+D31</f>
         <v>40570</v>
       </c>
-      <c r="E32" s="32" t="n">
+      <c r="E32" s="25" t="n">
         <f aca="false">E30+E31</f>
         <v>23845</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="8" t="s">
-        <v>115</v>
-      </c>
-      <c r="B33" s="32" t="n">
-        <f aca="false">MROUND(B32,Assumptions!$B$13)</f>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="7" t="s">
+        <v>112</v>
+      </c>
+      <c r="B33" s="25" t="n">
+        <f aca="false">CEILING(B32,Assumptions!$B$13)</f>
         <v>11500</v>
       </c>
-      <c r="C33" s="32" t="n">
-        <f aca="false">MROUND(C32,Assumptions!$B$13)</f>
-        <v>23750</v>
-      </c>
-      <c r="D33" s="32" t="n">
-        <f aca="false">MROUND(D32,Assumptions!$B$13)</f>
-        <v>40500</v>
-      </c>
-      <c r="E33" s="32" t="n">
-        <f aca="false">MROUND(E32,Assumptions!$B$13)</f>
-        <v>23750</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="8" t="s">
-        <v>116</v>
-      </c>
-      <c r="B35" s="32" t="n">
+      <c r="C33" s="25" t="n">
+        <f aca="false">CEILING(C32,Assumptions!$B$13)</f>
+        <v>23900</v>
+      </c>
+      <c r="D33" s="25" t="n">
+        <f aca="false">CEILING(D32,Assumptions!$B$13)</f>
+        <v>40600</v>
+      </c>
+      <c r="E33" s="25" t="n">
+        <f aca="false">CEILING(E32,Assumptions!$B$13)</f>
+        <v>23900</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="B35" s="25" t="n">
         <f aca="false">SUM(B33:D33)</f>
-        <v>75750</v>
-      </c>
-    </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="7" t="s">
-        <v>117</v>
+        <v>76000</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="6" t="s">
+        <v>114</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Restructure spreadsheet: tier columns as location-independent scenarios plus Program builder assigning changeable tiers to events
</commit_message>
<xml_diff>
--- a/pricing-model.xlsx
+++ b/pricing-model.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="123">
   <si>
     <t xml:space="preserve">AWS 1P Public Sector Symposiums - Pricing Model</t>
   </si>
@@ -30,16 +30,28 @@
     <t xml:space="preserve">This workbook mirrors pricing.config.js in the aws-1p-symposiums-proposal site. Same roles, rates, hour formulas, modifiers, and tier presets.</t>
   </si>
   <si>
+    <t xml:space="preserve">TWO INDEPENDENT AXES</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tiers (Lean, Signature, Premium) are service-level scenarios. They are not locations and are priced without reference to any event.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Symposiums (London, Ottawa, Canberra) are the three events. Each gets a tier ASSIGNED in the Program builder; the default is our recommendation based on readiness and is fully changeable.</t>
+  </si>
+  <si>
     <t xml:space="preserve">HOW TO USE</t>
   </si>
   <si>
     <t xml:space="preserve">Blue cells are inputs you can change. Black cells are formulas; do not overwrite them.</t>
   </si>
   <si>
-    <t xml:space="preserve">Assumptions sheet: rates, base hours by writing depth, modifiers, and tier presets. Edit blue values and the Calculator updates.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Calculator sheet: London, Ottawa, and Canberra pull their inputs from the tier presets (Lean / Signature / Premium). The Custom column is free-form.</t>
+    <t xml:space="preserve">Assumptions sheet: rates, base hours by writing depth, modifiers, tier presets, and symposium readiness notes.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Calculator sheet, top: each tier column prices one service-level scenario. The Custom column is free-form.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Calculator sheet, Program builder: pick a tier for each symposium (dropdown) and the program total sums the three.</t>
   </si>
   <si>
     <t xml:space="preserve">FEEDING CHANGES BACK TO THE SITE</t>
@@ -57,10 +69,10 @@
     <t xml:space="preserve">2. Modifiers add hours: slides above 20 add design time, each speaker adds speaker management, each edit round adds design and writing, each dry run adds PM and writing.</t>
   </si>
   <si>
-    <t xml:space="preserve">3. Cost = sum of role hours x rates, plus flat on-site day rate x days.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4. Headline prices round UP to the nearest $100. Program total = sum of the three rounded city prices.</t>
+    <t xml:space="preserve">3. Cost = sum of role hours x rates, plus flat on-site day rate x days (0 days = none).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4. Headline prices round UP to the nearest $100. Program total = sum of the three assigned per-deck prices.</t>
   </si>
   <si>
     <t xml:space="preserve">ALL NUMBERS ARE PLACEHOLDERS PENDING CONFIRMATION. Estimate, not a quote.</t>
@@ -228,10 +240,10 @@
     <t xml:space="preserve">modifiers.perDryRun.writing</t>
   </si>
   <si>
-    <t xml:space="preserve">Tier presets</t>
-  </si>
-  <si>
-    <t xml:space="preserve">On-site days of 0 means on-site support is off. Depth: 1 = Deck mods only, 2 = Scripting from framework, 3 = Full narrative + scripting.</t>
+    <t xml:space="preserve">Tier presets (service levels, independent of any event)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Depth: 1 = Deck mods only, 2 = Scripting from framework, 3 = Full narrative + scripting. On-site days of 0 = off.</t>
   </si>
   <si>
     <t xml:space="preserve">Tier</t>
@@ -273,10 +285,10 @@
     <t xml:space="preserve">tiers[premium].preset</t>
   </si>
   <si>
-    <t xml:space="preserve">Symposium readiness and recommended starting service level</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Recommendations only. The client confirmed the events and their readiness; the tier mapping is our suggestion and changeable on the Calculator.</t>
+    <t xml:space="preserve">Symposium readiness (events, independent of any tier)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The client confirmed the events and their readiness. The recommended tier is OUR suggested starting point and is changeable in the Program builder.</t>
   </si>
   <si>
     <t xml:space="preserve">Symposium</t>
@@ -315,10 +327,10 @@
     <t xml:space="preserve">symposiums[canberra].recommendedTier / .readiness</t>
   </si>
   <si>
-    <t xml:space="preserve">Per-Deck Pricing Calculator</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tiers are service levels, not locations: any symposium can run at any tier. The blue tier name per city defaults to OUR recommended starting point (based on readiness) and is fully changeable. Custom column is free-form. Headline prices round UP to the nearest \$100; the breakdown shows exact math. Estimate, not a quote.</t>
+    <t xml:space="preserve">Service-Level Pricing Scenarios</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Each column prices one TIER, independent of any event. Lean / Signature / Premium pull from the presets on Assumptions; Custom is free-form (blue). Assign tiers to events in the Program builder below. Estimate, not a quote.</t>
   </si>
   <si>
     <t xml:space="preserve">Custom</t>
@@ -363,10 +375,22 @@
     <t xml:space="preserve">Per-deck total (rounded up)</t>
   </si>
   <si>
-    <t xml:space="preserve">Program total (London + Ottawa + Canberra, rounded)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Custom column is a scratch scenario; it is not included in the program total.</t>
+    <t xml:space="preserve">Program Builder</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Assign a service level to each event. The selected tier defaults to our recommendation (readiness-based) and is changeable: any event can take any tier, including Custom.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Selected tier</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Per-deck price</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Program total</t>
+  </si>
+  <si>
+    <t xml:space="preserve">If multiple events select Custom, they share the single Custom scenario column above.</t>
   </si>
 </sst>
 </file>
@@ -378,7 +402,7 @@
     <numFmt numFmtId="165" formatCode="\$#,##0"/>
     <numFmt numFmtId="166" formatCode="0.##"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -451,6 +475,13 @@
       <family val="0"/>
       <charset val="1"/>
     </font>
+    <font>
+      <b val="true"/>
+      <sz val="12"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -512,7 +543,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="28">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -577,18 +608,14 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -615,6 +642,18 @@
     </xf>
     <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -869,7 +908,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:A18"/>
+  <dimension ref="A1:A23"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="110"/>
@@ -893,7 +932,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
         <v>3</v>
       </c>
@@ -903,58 +942,81 @@
         <v>4</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="2" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="2"/>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="3" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="2"/>
-    </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3" t="s">
+      <c r="A9" s="2" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="2"/>
+      <c r="A11" s="2" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="3" t="s">
-        <v>8</v>
+      <c r="A12" s="2" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="2" t="s">
+      <c r="A13" s="2"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="3" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="2" t="s">
+      <c r="A16" s="2"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="3" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="2"/>
-    </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="4" t="s">
+      <c r="A18" s="2" t="s">
         <v>13</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="2"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="4" t="s">
+        <v>17</v>
       </c>
     </row>
   </sheetData>
@@ -977,185 +1039,182 @@
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="2" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="2" style="0" width="16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="5" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="34"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="H5" s="8" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="9" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="B6" s="10" t="n">
         <v>185</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="H6" s="6" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="B7" s="10" t="n">
         <v>185</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="H7" s="6" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="9" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="B8" s="10" t="n">
         <v>175</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="H8" s="6" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="9" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="B9" s="10" t="n">
         <v>200</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="H9" s="6" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="9" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="B10" s="10" t="n">
         <v>175</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="H10" s="6" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="9" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="B11" s="10" t="n">
         <v>100</v>
       </c>
       <c r="C11" s="9" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="H11" s="6" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="9" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="B12" s="10" t="n">
         <v>3500</v>
       </c>
       <c r="C12" s="9" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="H12" s="6" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="9" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="B13" s="10" t="n">
         <v>100</v>
       </c>
       <c r="C13" s="9" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="H13" s="6" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="11" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="B18" s="11" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="C18" s="11" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="D18" s="11" t="s">
-        <v>44</v>
-      </c>
-      <c r="E18" s="11"/>
-      <c r="F18" s="11"/>
-      <c r="G18" s="11"/>
+        <v>48</v>
+      </c>
       <c r="H18" s="11" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="9" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="B19" s="12" t="n">
         <v>4</v>
@@ -1167,12 +1226,12 @@
         <v>48</v>
       </c>
       <c r="H19" s="6" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="9" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="B20" s="12" t="n">
         <v>0</v>
@@ -1184,12 +1243,12 @@
         <v>22</v>
       </c>
       <c r="H20" s="6" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="9" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="B21" s="12" t="n">
         <v>20</v>
@@ -1201,12 +1260,12 @@
         <v>20</v>
       </c>
       <c r="H21" s="6" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="9" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="B22" s="12" t="n">
         <v>3</v>
@@ -1218,12 +1277,12 @@
         <v>8</v>
       </c>
       <c r="H22" s="6" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="9" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="B23" s="12" t="n">
         <v>6</v>
@@ -1235,12 +1294,12 @@
         <v>6</v>
       </c>
       <c r="H23" s="6" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="9" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="B24" s="12" t="n">
         <v>5</v>
@@ -1252,141 +1311,141 @@
         <v>5</v>
       </c>
       <c r="H24" s="6" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="7" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="8" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="B28" s="8" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="H28" s="8" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="9" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="B29" s="12" t="n">
         <v>20</v>
       </c>
       <c r="H29" s="6" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="9" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="B30" s="12" t="n">
         <v>0.6</v>
       </c>
       <c r="H30" s="6" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="9" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="B31" s="12" t="n">
         <v>3</v>
       </c>
       <c r="H31" s="6" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="9" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="B32" s="12" t="n">
         <v>4</v>
       </c>
       <c r="H32" s="6" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="9" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="B33" s="12" t="n">
         <v>2</v>
       </c>
       <c r="H33" s="6" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="9" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="B34" s="12" t="n">
         <v>4</v>
       </c>
       <c r="H34" s="6" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="9" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="B35" s="12" t="n">
         <v>3</v>
       </c>
       <c r="H35" s="6" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="7" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="6" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="11" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="B40" s="11" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="C40" s="11" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="D40" s="11" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="E40" s="11" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="F40" s="11" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="G40" s="11" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="H40" s="11" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="9" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="B41" s="13" t="n">
         <v>20</v>
@@ -1407,12 +1466,12 @@
         <v>0</v>
       </c>
       <c r="H41" s="6" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="9" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="B42" s="13" t="n">
         <v>35</v>
@@ -1433,12 +1492,12 @@
         <v>1</v>
       </c>
       <c r="H42" s="6" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="9" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="B43" s="13" t="n">
         <v>50</v>
@@ -1459,73 +1518,73 @@
         <v>2</v>
       </c>
       <c r="H43" s="6" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="7" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="6" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="8" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="B47" s="8" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="C47" s="8" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="H47" s="8" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="9" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="B48" s="13" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="C48" s="9" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="H48" s="6" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="9" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="B49" s="13" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="C49" s="9" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="H49" s="6" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="9" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="B50" s="13" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="C50" s="9" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="H50" s="6" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
     </row>
   </sheetData>
@@ -1544,586 +1603,666 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E36"/>
+  <dimension ref="A1:E42"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="2" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="16"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="14" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="15"/>
       <c r="B4" s="15" t="s">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="C4" s="15" t="s">
-        <v>91</v>
+        <v>83</v>
       </c>
       <c r="D4" s="15" t="s">
-        <v>94</v>
+        <v>85</v>
       </c>
       <c r="E4" s="15" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="7" t="s">
-        <v>70</v>
-      </c>
-      <c r="B5" s="16" t="s">
-        <v>77</v>
-      </c>
-      <c r="C5" s="16" t="s">
-        <v>79</v>
-      </c>
-      <c r="D5" s="16" t="s">
-        <v>81</v>
-      </c>
-      <c r="E5" s="17" t="s">
-        <v>99</v>
+      <c r="A5" s="9" t="s">
+        <v>75</v>
+      </c>
+      <c r="B5" s="16" t="n">
+        <f aca="false">INDEX(Assumptions!$B$41:$B$43,MATCH(B$4,Assumptions!$A$41:$A$43,0))</f>
+        <v>20</v>
+      </c>
+      <c r="C5" s="16" t="n">
+        <f aca="false">INDEX(Assumptions!$B$41:$B$43,MATCH(C$4,Assumptions!$A$41:$A$43,0))</f>
+        <v>35</v>
+      </c>
+      <c r="D5" s="16" t="n">
+        <f aca="false">INDEX(Assumptions!$B$41:$B$43,MATCH(D$4,Assumptions!$A$41:$A$43,0))</f>
+        <v>50</v>
+      </c>
+      <c r="E5" s="17" t="n">
+        <v>35</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="9" t="s">
-        <v>71</v>
-      </c>
-      <c r="B6" s="18" t="n">
-        <f aca="false">INDEX(Assumptions!$B$41:$B$43,MATCH(B$5,Assumptions!$A$41:$A$43,0))</f>
-        <v>20</v>
-      </c>
-      <c r="C6" s="18" t="n">
-        <f aca="false">INDEX(Assumptions!$B$41:$B$43,MATCH(C$5,Assumptions!$A$41:$A$43,0))</f>
-        <v>35</v>
-      </c>
-      <c r="D6" s="18" t="n">
-        <f aca="false">INDEX(Assumptions!$B$41:$B$43,MATCH(D$5,Assumptions!$A$41:$A$43,0))</f>
-        <v>50</v>
-      </c>
-      <c r="E6" s="16" t="n">
-        <v>35</v>
+        <v>104</v>
+      </c>
+      <c r="B6" s="16" t="n">
+        <f aca="false">INDEX(Assumptions!$C$41:$C$43,MATCH(B$4,Assumptions!$A$41:$A$43,0))</f>
+        <v>1</v>
+      </c>
+      <c r="C6" s="16" t="n">
+        <f aca="false">INDEX(Assumptions!$C$41:$C$43,MATCH(C$4,Assumptions!$A$41:$A$43,0))</f>
+        <v>2</v>
+      </c>
+      <c r="D6" s="16" t="n">
+        <f aca="false">INDEX(Assumptions!$C$41:$C$43,MATCH(D$4,Assumptions!$A$41:$A$43,0))</f>
+        <v>3</v>
+      </c>
+      <c r="E6" s="17" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>100</v>
-      </c>
-      <c r="B7" s="18" t="n">
-        <f aca="false">INDEX(Assumptions!$C$41:$C$43,MATCH(B$5,Assumptions!$A$41:$A$43,0))</f>
-        <v>1</v>
-      </c>
-      <c r="C7" s="18" t="n">
-        <f aca="false">INDEX(Assumptions!$C$41:$C$43,MATCH(C$5,Assumptions!$A$41:$A$43,0))</f>
-        <v>2</v>
-      </c>
-      <c r="D7" s="18" t="n">
-        <f aca="false">INDEX(Assumptions!$C$41:$C$43,MATCH(D$5,Assumptions!$A$41:$A$43,0))</f>
-        <v>3</v>
-      </c>
-      <c r="E7" s="16" t="n">
-        <v>2</v>
+        <v>105</v>
+      </c>
+      <c r="B7" s="18" t="str">
+        <f aca="false">CHOOSE(B6,"Deck mods only","Scripting","Full narrative")</f>
+        <v>Deck mods only</v>
+      </c>
+      <c r="C7" s="18" t="str">
+        <f aca="false">CHOOSE(C6,"Deck mods only","Scripting","Full narrative")</f>
+        <v>Scripting</v>
+      </c>
+      <c r="D7" s="18" t="str">
+        <f aca="false">CHOOSE(D6,"Deck mods only","Scripting","Full narrative")</f>
+        <v>Full narrative</v>
+      </c>
+      <c r="E7" s="18" t="str">
+        <f aca="false">CHOOSE(E6,"Deck mods only","Scripting","Full narrative")</f>
+        <v>Scripting</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="9" t="s">
-        <v>101</v>
-      </c>
-      <c r="B8" s="19" t="str">
-        <f aca="false">CHOOSE(B7,"Deck mods only","Scripting","Full narrative")</f>
-        <v>Deck mods only</v>
-      </c>
-      <c r="C8" s="19" t="str">
-        <f aca="false">CHOOSE(C7,"Deck mods only","Scripting","Full narrative")</f>
-        <v>Scripting</v>
-      </c>
-      <c r="D8" s="19" t="str">
-        <f aca="false">CHOOSE(D7,"Deck mods only","Scripting","Full narrative")</f>
-        <v>Full narrative</v>
-      </c>
-      <c r="E8" s="19" t="str">
-        <f aca="false">CHOOSE(E7,"Deck mods only","Scripting","Full narrative")</f>
-        <v>Scripting</v>
+        <v>106</v>
+      </c>
+      <c r="B8" s="16" t="n">
+        <f aca="false">INDEX(Assumptions!$D$41:$D$43,MATCH(B$4,Assumptions!$A$41:$A$43,0))</f>
+        <v>3</v>
+      </c>
+      <c r="C8" s="16" t="n">
+        <f aca="false">INDEX(Assumptions!$D$41:$D$43,MATCH(C$4,Assumptions!$A$41:$A$43,0))</f>
+        <v>4</v>
+      </c>
+      <c r="D8" s="16" t="n">
+        <f aca="false">INDEX(Assumptions!$D$41:$D$43,MATCH(D$4,Assumptions!$A$41:$A$43,0))</f>
+        <v>5</v>
+      </c>
+      <c r="E8" s="17" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="9" t="s">
-        <v>102</v>
-      </c>
-      <c r="B9" s="18" t="n">
-        <f aca="false">INDEX(Assumptions!$D$41:$D$43,MATCH(B$5,Assumptions!$A$41:$A$43,0))</f>
+        <v>107</v>
+      </c>
+      <c r="B9" s="16" t="n">
+        <f aca="false">INDEX(Assumptions!$E$41:$E$43,MATCH(B$4,Assumptions!$A$41:$A$43,0))</f>
+        <v>2</v>
+      </c>
+      <c r="C9" s="16" t="n">
+        <f aca="false">INDEX(Assumptions!$E$41:$E$43,MATCH(C$4,Assumptions!$A$41:$A$43,0))</f>
         <v>3</v>
       </c>
-      <c r="C9" s="18" t="n">
-        <f aca="false">INDEX(Assumptions!$D$41:$D$43,MATCH(C$5,Assumptions!$A$41:$A$43,0))</f>
+      <c r="D9" s="16" t="n">
+        <f aca="false">INDEX(Assumptions!$E$41:$E$43,MATCH(D$4,Assumptions!$A$41:$A$43,0))</f>
         <v>4</v>
       </c>
-      <c r="D9" s="18" t="n">
-        <f aca="false">INDEX(Assumptions!$D$41:$D$43,MATCH(D$5,Assumptions!$A$41:$A$43,0))</f>
-        <v>5</v>
-      </c>
-      <c r="E9" s="16" t="n">
-        <v>4</v>
+      <c r="E9" s="17" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="9" t="s">
-        <v>103</v>
-      </c>
-      <c r="B10" s="18" t="n">
-        <f aca="false">INDEX(Assumptions!$E$41:$E$43,MATCH(B$5,Assumptions!$A$41:$A$43,0))</f>
+        <v>108</v>
+      </c>
+      <c r="B10" s="16" t="n">
+        <f aca="false">INDEX(Assumptions!$F$41:$F$43,MATCH(B$4,Assumptions!$A$41:$A$43,0))</f>
+        <v>1</v>
+      </c>
+      <c r="C10" s="16" t="n">
+        <f aca="false">INDEX(Assumptions!$F$41:$F$43,MATCH(C$4,Assumptions!$A$41:$A$43,0))</f>
         <v>2</v>
       </c>
-      <c r="C10" s="18" t="n">
-        <f aca="false">INDEX(Assumptions!$E$41:$E$43,MATCH(C$5,Assumptions!$A$41:$A$43,0))</f>
+      <c r="D10" s="16" t="n">
+        <f aca="false">INDEX(Assumptions!$F$41:$F$43,MATCH(D$4,Assumptions!$A$41:$A$43,0))</f>
         <v>3</v>
       </c>
-      <c r="D10" s="18" t="n">
-        <f aca="false">INDEX(Assumptions!$E$41:$E$43,MATCH(D$5,Assumptions!$A$41:$A$43,0))</f>
-        <v>4</v>
-      </c>
-      <c r="E10" s="16" t="n">
-        <v>3</v>
+      <c r="E10" s="17" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="9" t="s">
-        <v>104</v>
-      </c>
-      <c r="B11" s="18" t="n">
-        <f aca="false">INDEX(Assumptions!$F$41:$F$43,MATCH(B$5,Assumptions!$A$41:$A$43,0))</f>
+        <v>109</v>
+      </c>
+      <c r="B11" s="16" t="n">
+        <f aca="false">INDEX(Assumptions!$G$41:$G$43,MATCH(B$4,Assumptions!$A$41:$A$43,0))</f>
+        <v>0</v>
+      </c>
+      <c r="C11" s="16" t="n">
+        <f aca="false">INDEX(Assumptions!$G$41:$G$43,MATCH(C$4,Assumptions!$A$41:$A$43,0))</f>
         <v>1</v>
       </c>
-      <c r="C11" s="18" t="n">
-        <f aca="false">INDEX(Assumptions!$F$41:$F$43,MATCH(C$5,Assumptions!$A$41:$A$43,0))</f>
+      <c r="D11" s="16" t="n">
+        <f aca="false">INDEX(Assumptions!$G$41:$G$43,MATCH(D$4,Assumptions!$A$41:$A$43,0))</f>
         <v>2</v>
       </c>
-      <c r="D11" s="18" t="n">
-        <f aca="false">INDEX(Assumptions!$F$41:$F$43,MATCH(D$5,Assumptions!$A$41:$A$43,0))</f>
-        <v>3</v>
-      </c>
-      <c r="E11" s="16" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="9" t="s">
-        <v>105</v>
-      </c>
-      <c r="B12" s="18" t="n">
-        <f aca="false">INDEX(Assumptions!$G$41:$G$43,MATCH(B$5,Assumptions!$A$41:$A$43,0))</f>
-        <v>0</v>
-      </c>
-      <c r="C12" s="18" t="n">
-        <f aca="false">INDEX(Assumptions!$G$41:$G$43,MATCH(C$5,Assumptions!$A$41:$A$43,0))</f>
+      <c r="E11" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="D12" s="18" t="n">
-        <f aca="false">INDEX(Assumptions!$G$41:$G$43,MATCH(D$5,Assumptions!$A$41:$A$43,0))</f>
-        <v>2</v>
-      </c>
-      <c r="E12" s="16" t="n">
-        <v>1</v>
-      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="19" t="s">
+        <v>110</v>
+      </c>
+      <c r="B13" s="20"/>
+      <c r="C13" s="20"/>
+      <c r="D13" s="20"/>
+      <c r="E13" s="20"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="20" t="s">
-        <v>106</v>
-      </c>
-      <c r="B14" s="21"/>
-      <c r="C14" s="21"/>
-      <c r="D14" s="21"/>
-      <c r="E14" s="21"/>
+      <c r="A14" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="B14" s="21" t="n">
+        <f aca="false">INDEX(Assumptions!$B$19:$D$19,B6)+Assumptions!$B$33*B9+Assumptions!$B$35*B10</f>
+        <v>11</v>
+      </c>
+      <c r="C14" s="21" t="n">
+        <f aca="false">INDEX(Assumptions!$B$19:$D$19,C6)+Assumptions!$B$33*C9+Assumptions!$B$35*C10</f>
+        <v>32</v>
+      </c>
+      <c r="D14" s="21" t="n">
+        <f aca="false">INDEX(Assumptions!$B$19:$D$19,D6)+Assumptions!$B$33*D9+Assumptions!$B$35*D10</f>
+        <v>65</v>
+      </c>
+      <c r="E14" s="21" t="n">
+        <f aca="false">INDEX(Assumptions!$B$19:$D$19,E6)+Assumptions!$B$33*E9+Assumptions!$B$35*E10</f>
+        <v>32</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="B15" s="22" t="n">
-        <f aca="false">INDEX(Assumptions!$B$19:$D$19,B7)+Assumptions!$B$33*B10+Assumptions!$B$35*B11</f>
-        <v>11</v>
-      </c>
-      <c r="C15" s="22" t="n">
-        <f aca="false">INDEX(Assumptions!$B$19:$D$19,C7)+Assumptions!$B$33*C10+Assumptions!$B$35*C11</f>
-        <v>32</v>
-      </c>
-      <c r="D15" s="22" t="n">
-        <f aca="false">INDEX(Assumptions!$B$19:$D$19,D7)+Assumptions!$B$33*D10+Assumptions!$B$35*D11</f>
-        <v>65</v>
-      </c>
-      <c r="E15" s="22" t="n">
-        <f aca="false">INDEX(Assumptions!$B$19:$D$19,E7)+Assumptions!$B$33*E10+Assumptions!$B$35*E11</f>
-        <v>32</v>
+        <v>28</v>
+      </c>
+      <c r="B15" s="21" t="n">
+        <f aca="false">INDEX(Assumptions!$B$20:$D$20,B6)+Assumptions!$B$31*B8</f>
+        <v>9</v>
+      </c>
+      <c r="C15" s="21" t="n">
+        <f aca="false">INDEX(Assumptions!$B$20:$D$20,C6)+Assumptions!$B$31*C8</f>
+        <v>20</v>
+      </c>
+      <c r="D15" s="21" t="n">
+        <f aca="false">INDEX(Assumptions!$B$20:$D$20,D6)+Assumptions!$B$31*D8</f>
+        <v>37</v>
+      </c>
+      <c r="E15" s="21" t="n">
+        <f aca="false">INDEX(Assumptions!$B$20:$D$20,E6)+Assumptions!$B$31*E8</f>
+        <v>20</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="9" t="s">
-        <v>24</v>
-      </c>
-      <c r="B16" s="22" t="n">
-        <f aca="false">INDEX(Assumptions!$B$20:$D$20,B7)+Assumptions!$B$31*B9</f>
-        <v>9</v>
-      </c>
-      <c r="C16" s="22" t="n">
-        <f aca="false">INDEX(Assumptions!$B$20:$D$20,C7)+Assumptions!$B$31*C9</f>
-        <v>20</v>
-      </c>
-      <c r="D16" s="22" t="n">
-        <f aca="false">INDEX(Assumptions!$B$20:$D$20,D7)+Assumptions!$B$31*D9</f>
-        <v>37</v>
-      </c>
-      <c r="E16" s="22" t="n">
-        <f aca="false">INDEX(Assumptions!$B$20:$D$20,E7)+Assumptions!$B$31*E9</f>
-        <v>20</v>
+        <v>30</v>
+      </c>
+      <c r="B16" s="21" t="n">
+        <f aca="false">INDEX(Assumptions!$B$21:$D$21,B6)+Assumptions!$B$30*MAX(0,B5-Assumptions!$B$29)+Assumptions!$B$32*B9</f>
+        <v>28</v>
+      </c>
+      <c r="C16" s="21" t="n">
+        <f aca="false">INDEX(Assumptions!$B$21:$D$21,C6)+Assumptions!$B$30*MAX(0,C5-Assumptions!$B$29)+Assumptions!$B$32*C9</f>
+        <v>41</v>
+      </c>
+      <c r="D16" s="21" t="n">
+        <f aca="false">INDEX(Assumptions!$B$21:$D$21,D6)+Assumptions!$B$30*MAX(0,D5-Assumptions!$B$29)+Assumptions!$B$32*D9</f>
+        <v>54</v>
+      </c>
+      <c r="E16" s="21" t="n">
+        <f aca="false">INDEX(Assumptions!$B$21:$D$21,E6)+Assumptions!$B$30*MAX(0,E5-Assumptions!$B$29)+Assumptions!$B$32*E9</f>
+        <v>41</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="B17" s="22" t="n">
-        <f aca="false">INDEX(Assumptions!$B$21:$D$21,B7)+Assumptions!$B$30*MAX(0,B6-Assumptions!$B$29)+Assumptions!$B$32*B10</f>
-        <v>28</v>
-      </c>
-      <c r="C17" s="22" t="n">
-        <f aca="false">INDEX(Assumptions!$B$21:$D$21,C7)+Assumptions!$B$30*MAX(0,C6-Assumptions!$B$29)+Assumptions!$B$32*C10</f>
-        <v>41</v>
-      </c>
-      <c r="D17" s="22" t="n">
-        <f aca="false">INDEX(Assumptions!$B$21:$D$21,D7)+Assumptions!$B$30*MAX(0,D6-Assumptions!$B$29)+Assumptions!$B$32*D10</f>
-        <v>54</v>
-      </c>
-      <c r="E17" s="22" t="n">
-        <f aca="false">INDEX(Assumptions!$B$21:$D$21,E7)+Assumptions!$B$30*MAX(0,E6-Assumptions!$B$29)+Assumptions!$B$32*E10</f>
-        <v>41</v>
+        <v>32</v>
+      </c>
+      <c r="B17" s="21" t="n">
+        <f aca="false">INDEX(Assumptions!$B$22:$D$22,B6)</f>
+        <v>3</v>
+      </c>
+      <c r="C17" s="21" t="n">
+        <f aca="false">INDEX(Assumptions!$B$22:$D$22,C6)</f>
+        <v>3</v>
+      </c>
+      <c r="D17" s="21" t="n">
+        <f aca="false">INDEX(Assumptions!$B$22:$D$22,D6)</f>
+        <v>8</v>
+      </c>
+      <c r="E17" s="21" t="n">
+        <f aca="false">INDEX(Assumptions!$B$22:$D$22,E6)</f>
+        <v>3</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="B18" s="22" t="n">
-        <f aca="false">INDEX(Assumptions!$B$22:$D$22,B7)</f>
-        <v>3</v>
-      </c>
-      <c r="C18" s="22" t="n">
-        <f aca="false">INDEX(Assumptions!$B$22:$D$22,C7)</f>
-        <v>3</v>
-      </c>
-      <c r="D18" s="22" t="n">
-        <f aca="false">INDEX(Assumptions!$B$22:$D$22,D7)</f>
-        <v>8</v>
-      </c>
-      <c r="E18" s="22" t="n">
-        <f aca="false">INDEX(Assumptions!$B$22:$D$22,E7)</f>
-        <v>3</v>
+        <v>34</v>
+      </c>
+      <c r="B18" s="21" t="n">
+        <f aca="false">INDEX(Assumptions!$B$23:$D$23,B6)+Assumptions!$B$34*B10</f>
+        <v>10</v>
+      </c>
+      <c r="C18" s="21" t="n">
+        <f aca="false">INDEX(Assumptions!$B$23:$D$23,C6)+Assumptions!$B$34*C10</f>
+        <v>14</v>
+      </c>
+      <c r="D18" s="21" t="n">
+        <f aca="false">INDEX(Assumptions!$B$23:$D$23,D6)+Assumptions!$B$34*D10</f>
+        <v>18</v>
+      </c>
+      <c r="E18" s="21" t="n">
+        <f aca="false">INDEX(Assumptions!$B$23:$D$23,E6)+Assumptions!$B$34*E10</f>
+        <v>14</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="9" t="s">
-        <v>30</v>
-      </c>
-      <c r="B19" s="22" t="n">
-        <f aca="false">INDEX(Assumptions!$B$23:$D$23,B7)+Assumptions!$B$34*B11</f>
-        <v>10</v>
-      </c>
-      <c r="C19" s="22" t="n">
-        <f aca="false">INDEX(Assumptions!$B$23:$D$23,C7)+Assumptions!$B$34*C11</f>
-        <v>14</v>
-      </c>
-      <c r="D19" s="22" t="n">
-        <f aca="false">INDEX(Assumptions!$B$23:$D$23,D7)+Assumptions!$B$34*D11</f>
-        <v>18</v>
-      </c>
-      <c r="E19" s="22" t="n">
-        <f aca="false">INDEX(Assumptions!$B$23:$D$23,E7)+Assumptions!$B$34*E11</f>
-        <v>14</v>
+        <v>36</v>
+      </c>
+      <c r="B19" s="21" t="n">
+        <f aca="false">INDEX(Assumptions!$B$24:$D$24,B6)</f>
+        <v>5</v>
+      </c>
+      <c r="C19" s="21" t="n">
+        <f aca="false">INDEX(Assumptions!$B$24:$D$24,C6)</f>
+        <v>5</v>
+      </c>
+      <c r="D19" s="21" t="n">
+        <f aca="false">INDEX(Assumptions!$B$24:$D$24,D6)</f>
+        <v>5</v>
+      </c>
+      <c r="E19" s="21" t="n">
+        <f aca="false">INDEX(Assumptions!$B$24:$D$24,E6)</f>
+        <v>5</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="9" t="s">
-        <v>32</v>
+      <c r="A20" s="7" t="s">
+        <v>111</v>
       </c>
       <c r="B20" s="22" t="n">
-        <f aca="false">INDEX(Assumptions!$B$24:$D$24,B7)</f>
-        <v>5</v>
+        <f aca="false">SUM(B14:B19)</f>
+        <v>66</v>
       </c>
       <c r="C20" s="22" t="n">
-        <f aca="false">INDEX(Assumptions!$B$24:$D$24,C7)</f>
-        <v>5</v>
+        <f aca="false">SUM(C14:C19)</f>
+        <v>115</v>
       </c>
       <c r="D20" s="22" t="n">
-        <f aca="false">INDEX(Assumptions!$B$24:$D$24,D7)</f>
-        <v>5</v>
+        <f aca="false">SUM(D14:D19)</f>
+        <v>187</v>
       </c>
       <c r="E20" s="22" t="n">
-        <f aca="false">INDEX(Assumptions!$B$24:$D$24,E7)</f>
-        <v>5</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="7" t="s">
-        <v>107</v>
-      </c>
-      <c r="B21" s="23" t="n">
-        <f aca="false">SUM(B15:B20)</f>
-        <v>66</v>
-      </c>
-      <c r="C21" s="23" t="n">
-        <f aca="false">SUM(C15:C20)</f>
+        <f aca="false">SUM(E14:E19)</f>
         <v>115</v>
       </c>
-      <c r="D21" s="23" t="n">
-        <f aca="false">SUM(D15:D20)</f>
-        <v>187</v>
-      </c>
-      <c r="E21" s="23" t="n">
-        <f aca="false">SUM(E15:E20)</f>
-        <v>115</v>
-      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="19" t="s">
+        <v>112</v>
+      </c>
+      <c r="B22" s="20"/>
+      <c r="C22" s="20"/>
+      <c r="D22" s="20"/>
+      <c r="E22" s="20"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="20" t="s">
-        <v>108</v>
-      </c>
-      <c r="B23" s="21"/>
-      <c r="C23" s="21"/>
-      <c r="D23" s="21"/>
-      <c r="E23" s="21"/>
+      <c r="A23" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="B23" s="23" t="n">
+        <f aca="false">B14*Assumptions!$B$6</f>
+        <v>2035</v>
+      </c>
+      <c r="C23" s="23" t="n">
+        <f aca="false">C14*Assumptions!$B$6</f>
+        <v>5920</v>
+      </c>
+      <c r="D23" s="23" t="n">
+        <f aca="false">D14*Assumptions!$B$6</f>
+        <v>12025</v>
+      </c>
+      <c r="E23" s="23" t="n">
+        <f aca="false">E14*Assumptions!$B$6</f>
+        <v>5920</v>
+      </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="B24" s="24" t="n">
-        <f aca="false">B15*Assumptions!$B$6</f>
-        <v>2035</v>
-      </c>
-      <c r="C24" s="24" t="n">
-        <f aca="false">C15*Assumptions!$B$6</f>
-        <v>5920</v>
-      </c>
-      <c r="D24" s="24" t="n">
-        <f aca="false">D15*Assumptions!$B$6</f>
-        <v>12025</v>
-      </c>
-      <c r="E24" s="24" t="n">
-        <f aca="false">E15*Assumptions!$B$6</f>
-        <v>5920</v>
+        <v>28</v>
+      </c>
+      <c r="B24" s="23" t="n">
+        <f aca="false">B15*Assumptions!$B$7</f>
+        <v>1665</v>
+      </c>
+      <c r="C24" s="23" t="n">
+        <f aca="false">C15*Assumptions!$B$7</f>
+        <v>3700</v>
+      </c>
+      <c r="D24" s="23" t="n">
+        <f aca="false">D15*Assumptions!$B$7</f>
+        <v>6845</v>
+      </c>
+      <c r="E24" s="23" t="n">
+        <f aca="false">E15*Assumptions!$B$7</f>
+        <v>3700</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="9" t="s">
-        <v>24</v>
-      </c>
-      <c r="B25" s="24" t="n">
-        <f aca="false">B16*Assumptions!$B$7</f>
-        <v>1665</v>
-      </c>
-      <c r="C25" s="24" t="n">
-        <f aca="false">C16*Assumptions!$B$7</f>
-        <v>3700</v>
-      </c>
-      <c r="D25" s="24" t="n">
-        <f aca="false">D16*Assumptions!$B$7</f>
-        <v>6845</v>
-      </c>
-      <c r="E25" s="24" t="n">
-        <f aca="false">E16*Assumptions!$B$7</f>
-        <v>3700</v>
+        <v>30</v>
+      </c>
+      <c r="B25" s="23" t="n">
+        <f aca="false">B16*Assumptions!$B$8</f>
+        <v>4900</v>
+      </c>
+      <c r="C25" s="23" t="n">
+        <f aca="false">C16*Assumptions!$B$8</f>
+        <v>7175</v>
+      </c>
+      <c r="D25" s="23" t="n">
+        <f aca="false">D16*Assumptions!$B$8</f>
+        <v>9450</v>
+      </c>
+      <c r="E25" s="23" t="n">
+        <f aca="false">E16*Assumptions!$B$8</f>
+        <v>7175</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="B26" s="24" t="n">
-        <f aca="false">B17*Assumptions!$B$8</f>
-        <v>4900</v>
-      </c>
-      <c r="C26" s="24" t="n">
-        <f aca="false">C17*Assumptions!$B$8</f>
-        <v>7175</v>
-      </c>
-      <c r="D26" s="24" t="n">
-        <f aca="false">D17*Assumptions!$B$8</f>
-        <v>9450</v>
-      </c>
-      <c r="E26" s="24" t="n">
-        <f aca="false">E17*Assumptions!$B$8</f>
-        <v>7175</v>
+        <v>32</v>
+      </c>
+      <c r="B26" s="23" t="n">
+        <f aca="false">B17*Assumptions!$B$9</f>
+        <v>600</v>
+      </c>
+      <c r="C26" s="23" t="n">
+        <f aca="false">C17*Assumptions!$B$9</f>
+        <v>600</v>
+      </c>
+      <c r="D26" s="23" t="n">
+        <f aca="false">D17*Assumptions!$B$9</f>
+        <v>1600</v>
+      </c>
+      <c r="E26" s="23" t="n">
+        <f aca="false">E17*Assumptions!$B$9</f>
+        <v>600</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="B27" s="24" t="n">
-        <f aca="false">B18*Assumptions!$B$9</f>
-        <v>600</v>
-      </c>
-      <c r="C27" s="24" t="n">
-        <f aca="false">C18*Assumptions!$B$9</f>
-        <v>600</v>
-      </c>
-      <c r="D27" s="24" t="n">
-        <f aca="false">D18*Assumptions!$B$9</f>
-        <v>1600</v>
-      </c>
-      <c r="E27" s="24" t="n">
-        <f aca="false">E18*Assumptions!$B$9</f>
-        <v>600</v>
+        <v>34</v>
+      </c>
+      <c r="B27" s="23" t="n">
+        <f aca="false">B18*Assumptions!$B$10</f>
+        <v>1750</v>
+      </c>
+      <c r="C27" s="23" t="n">
+        <f aca="false">C18*Assumptions!$B$10</f>
+        <v>2450</v>
+      </c>
+      <c r="D27" s="23" t="n">
+        <f aca="false">D18*Assumptions!$B$10</f>
+        <v>3150</v>
+      </c>
+      <c r="E27" s="23" t="n">
+        <f aca="false">E18*Assumptions!$B$10</f>
+        <v>2450</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="9" t="s">
-        <v>30</v>
-      </c>
-      <c r="B28" s="24" t="n">
-        <f aca="false">B19*Assumptions!$B$10</f>
-        <v>1750</v>
-      </c>
-      <c r="C28" s="24" t="n">
-        <f aca="false">C19*Assumptions!$B$10</f>
-        <v>2450</v>
-      </c>
-      <c r="D28" s="24" t="n">
-        <f aca="false">D19*Assumptions!$B$10</f>
-        <v>3150</v>
-      </c>
-      <c r="E28" s="24" t="n">
-        <f aca="false">E19*Assumptions!$B$10</f>
-        <v>2450</v>
+        <v>36</v>
+      </c>
+      <c r="B28" s="23" t="n">
+        <f aca="false">B19*Assumptions!$B$11</f>
+        <v>500</v>
+      </c>
+      <c r="C28" s="23" t="n">
+        <f aca="false">C19*Assumptions!$B$11</f>
+        <v>500</v>
+      </c>
+      <c r="D28" s="23" t="n">
+        <f aca="false">D19*Assumptions!$B$11</f>
+        <v>500</v>
+      </c>
+      <c r="E28" s="23" t="n">
+        <f aca="false">E19*Assumptions!$B$11</f>
+        <v>500</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="9" t="s">
-        <v>32</v>
+      <c r="A29" s="7" t="s">
+        <v>113</v>
       </c>
       <c r="B29" s="24" t="n">
-        <f aca="false">B20*Assumptions!$B$11</f>
-        <v>500</v>
+        <f aca="false">SUM(B23:B28)</f>
+        <v>11450</v>
       </c>
       <c r="C29" s="24" t="n">
-        <f aca="false">C20*Assumptions!$B$11</f>
-        <v>500</v>
+        <f aca="false">SUM(C23:C28)</f>
+        <v>20345</v>
       </c>
       <c r="D29" s="24" t="n">
-        <f aca="false">D20*Assumptions!$B$11</f>
-        <v>500</v>
+        <f aca="false">SUM(D23:D28)</f>
+        <v>33570</v>
       </c>
       <c r="E29" s="24" t="n">
-        <f aca="false">E20*Assumptions!$B$11</f>
-        <v>500</v>
+        <f aca="false">SUM(E23:E28)</f>
+        <v>20345</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="7" t="s">
-        <v>109</v>
-      </c>
-      <c r="B30" s="25" t="n">
-        <f aca="false">SUM(B24:B29)</f>
+      <c r="A30" s="9" t="s">
+        <v>114</v>
+      </c>
+      <c r="B30" s="23" t="n">
+        <f aca="false">B11*Assumptions!$B$12</f>
+        <v>0</v>
+      </c>
+      <c r="C30" s="23" t="n">
+        <f aca="false">C11*Assumptions!$B$12</f>
+        <v>3500</v>
+      </c>
+      <c r="D30" s="23" t="n">
+        <f aca="false">D11*Assumptions!$B$12</f>
+        <v>7000</v>
+      </c>
+      <c r="E30" s="23" t="n">
+        <f aca="false">E11*Assumptions!$B$12</f>
+        <v>3500</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="7" t="s">
+        <v>115</v>
+      </c>
+      <c r="B31" s="24" t="n">
+        <f aca="false">B29+B30</f>
         <v>11450</v>
       </c>
-      <c r="C30" s="25" t="n">
-        <f aca="false">SUM(C24:C29)</f>
-        <v>20345</v>
-      </c>
-      <c r="D30" s="25" t="n">
-        <f aca="false">SUM(D24:D29)</f>
-        <v>33570</v>
-      </c>
-      <c r="E30" s="25" t="n">
-        <f aca="false">SUM(E24:E29)</f>
-        <v>20345</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="9" t="s">
-        <v>110</v>
-      </c>
-      <c r="B31" s="24" t="n">
-        <f aca="false">B12*Assumptions!$B$12</f>
-        <v>0</v>
-      </c>
       <c r="C31" s="24" t="n">
-        <f aca="false">C12*Assumptions!$B$12</f>
-        <v>3500</v>
+        <f aca="false">C29+C30</f>
+        <v>23845</v>
       </c>
       <c r="D31" s="24" t="n">
-        <f aca="false">D12*Assumptions!$B$12</f>
-        <v>7000</v>
+        <f aca="false">D29+D30</f>
+        <v>40570</v>
       </c>
       <c r="E31" s="24" t="n">
-        <f aca="false">E12*Assumptions!$B$12</f>
-        <v>3500</v>
+        <f aca="false">E29+E30</f>
+        <v>23845</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="7" t="s">
-        <v>111</v>
-      </c>
-      <c r="B32" s="25" t="n">
-        <f aca="false">B30+B31</f>
-        <v>11450</v>
-      </c>
-      <c r="C32" s="25" t="n">
-        <f aca="false">C30+C31</f>
-        <v>23845</v>
-      </c>
-      <c r="D32" s="25" t="n">
-        <f aca="false">D30+D31</f>
-        <v>40570</v>
-      </c>
-      <c r="E32" s="25" t="n">
-        <f aca="false">E30+E31</f>
-        <v>23845</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="7" t="s">
-        <v>112</v>
-      </c>
-      <c r="B33" s="25" t="n">
-        <f aca="false">CEILING(B32,Assumptions!$B$13)</f>
+        <v>116</v>
+      </c>
+      <c r="B32" s="24" t="n">
+        <f aca="false">CEILING(B31,Assumptions!$B$13)</f>
         <v>11500</v>
       </c>
-      <c r="C33" s="25" t="n">
-        <f aca="false">CEILING(C32,Assumptions!$B$13)</f>
+      <c r="C32" s="24" t="n">
+        <f aca="false">CEILING(C31,Assumptions!$B$13)</f>
         <v>23900</v>
       </c>
-      <c r="D33" s="25" t="n">
-        <f aca="false">CEILING(D32,Assumptions!$B$13)</f>
+      <c r="D32" s="24" t="n">
+        <f aca="false">CEILING(D31,Assumptions!$B$13)</f>
         <v>40600</v>
       </c>
-      <c r="E33" s="25" t="n">
-        <f aca="false">CEILING(E32,Assumptions!$B$13)</f>
+      <c r="E32" s="24" t="n">
+        <f aca="false">CEILING(E31,Assumptions!$B$13)</f>
         <v>23900</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="7" t="s">
-        <v>113</v>
-      </c>
-      <c r="B35" s="25" t="n">
-        <f aca="false">SUM(B33:D33)</f>
+      <c r="A35" s="25" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="14" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="11" t="s">
+        <v>89</v>
+      </c>
+      <c r="B37" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="C37" s="11" t="s">
+        <v>90</v>
+      </c>
+      <c r="D37" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="E37" s="11" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="26" t="str">
+        <f aca="false">Assumptions!A48</f>
+        <v>London</v>
+      </c>
+      <c r="B38" s="27" t="str">
+        <f aca="false">Assumptions!C48</f>
+        <v>Content is already written</v>
+      </c>
+      <c r="C38" s="26" t="str">
+        <f aca="false">Assumptions!B48</f>
+        <v>Lean</v>
+      </c>
+      <c r="D38" s="17" t="s">
+        <v>81</v>
+      </c>
+      <c r="E38" s="23" t="n">
+        <f aca="false">INDEX($B$32:$E$32,MATCH(D38,$B$4:$E$4,0))</f>
+        <v>11500</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="26" t="str">
+        <f aca="false">Assumptions!A49</f>
+        <v>Ottawa</v>
+      </c>
+      <c r="B39" s="27" t="str">
+        <f aca="false">Assumptions!C49</f>
+        <v>Owner in place; story still needs writing</v>
+      </c>
+      <c r="C39" s="26" t="str">
+        <f aca="false">Assumptions!B49</f>
+        <v>Signature</v>
+      </c>
+      <c r="D39" s="17" t="s">
+        <v>83</v>
+      </c>
+      <c r="E39" s="23" t="n">
+        <f aca="false">INDEX($B$32:$E$32,MATCH(D39,$B$4:$E$4,0))</f>
+        <v>23900</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="26" t="str">
+        <f aca="false">Assumptions!A50</f>
+        <v>Canberra</v>
+      </c>
+      <c r="B40" s="27" t="str">
+        <f aca="false">Assumptions!C50</f>
+        <v>Starting from scratch</v>
+      </c>
+      <c r="C40" s="26" t="str">
+        <f aca="false">Assumptions!B50</f>
+        <v>Premium</v>
+      </c>
+      <c r="D40" s="17" t="s">
+        <v>85</v>
+      </c>
+      <c r="E40" s="23" t="n">
+        <f aca="false">INDEX($B$32:$E$32,MATCH(D40,$B$4:$E$4,0))</f>
+        <v>40600</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="E41" s="24" t="n">
+        <f aca="false">SUM(E38:E40)</f>
         <v>76000</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="6" t="s">
-        <v>114</v>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="6" t="s">
+        <v>122</v>
       </c>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="D38:D40" type="list">
+      <formula1>"Lean,Signature,Premium,Custom"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+  </dataValidations>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>

<commit_message>
Sync team pricing round 2: Writing rate 250, on-site day rate 3000, writing hours 6/24/48 by depth
</commit_message>
<xml_diff>
--- a/pricing-model.xlsx
+++ b/pricing-model.xlsx
@@ -554,10 +554,10 @@
       <alignment shrinkToFit="0" vertical="bottom" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="7" numFmtId="165" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment vertical="bottom"/>
+      <alignment readingOrder="0" vertical="bottom"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="7" numFmtId="165" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0" vertical="bottom"/>
+      <alignment vertical="bottom"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="bottom"/>
@@ -3995,7 +3995,7 @@
         <v>25</v>
       </c>
       <c r="B6" s="11">
-        <v>200.0</v>
+        <v>250.0</v>
       </c>
       <c r="C6" s="10" t="s">
         <v>26</v>
@@ -4102,8 +4102,8 @@
       <c r="A12" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="B12" s="12">
-        <v>3500.0</v>
+      <c r="B12" s="11">
+        <v>3000.0</v>
       </c>
       <c r="C12" s="10" t="s">
         <v>39</v>
@@ -4203,12 +4203,12 @@
         <v>25</v>
       </c>
       <c r="B19" s="14">
-        <v>4.0</v>
+        <v>6.0</v>
       </c>
       <c r="C19" s="14">
-        <v>20.0</v>
-      </c>
-      <c r="D19" s="14">
+        <v>24.0</v>
+      </c>
+      <c r="D19" s="15">
         <v>48.0</v>
       </c>
       <c r="E19" s="5"/>
@@ -4222,13 +4222,13 @@
       <c r="A20" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="B20" s="15">
+      <c r="B20" s="14">
         <v>2.0</v>
       </c>
-      <c r="C20" s="14">
+      <c r="C20" s="15">
         <v>8.0</v>
       </c>
-      <c r="D20" s="14">
+      <c r="D20" s="15">
         <v>22.0</v>
       </c>
       <c r="E20" s="5"/>
@@ -4242,13 +4242,13 @@
       <c r="A21" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="B21" s="14">
+      <c r="B21" s="15">
         <v>20.0</v>
       </c>
-      <c r="C21" s="14">
+      <c r="C21" s="15">
         <v>20.0</v>
       </c>
-      <c r="D21" s="14">
+      <c r="D21" s="15">
         <v>20.0</v>
       </c>
       <c r="E21" s="5"/>
@@ -4262,13 +4262,13 @@
       <c r="A22" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="B22" s="14">
+      <c r="B22" s="15">
         <v>3.0</v>
       </c>
-      <c r="C22" s="14">
+      <c r="C22" s="15">
         <v>3.0</v>
       </c>
-      <c r="D22" s="14">
+      <c r="D22" s="15">
         <v>8.0</v>
       </c>
       <c r="E22" s="5"/>
@@ -4282,13 +4282,13 @@
       <c r="A23" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="B23" s="14">
+      <c r="B23" s="15">
         <v>6.0</v>
       </c>
-      <c r="C23" s="15">
+      <c r="C23" s="14">
         <v>8.0</v>
       </c>
-      <c r="D23" s="15">
+      <c r="D23" s="14">
         <v>10.0</v>
       </c>
       <c r="E23" s="5"/>
@@ -4302,13 +4302,13 @@
       <c r="A24" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="B24" s="14">
+      <c r="B24" s="15">
         <v>5.0</v>
       </c>
-      <c r="C24" s="15">
+      <c r="C24" s="14">
         <v>6.0</v>
       </c>
-      <c r="D24" s="15">
+      <c r="D24" s="14">
         <v>7.0</v>
       </c>
       <c r="E24" s="5"/>
@@ -4370,7 +4370,7 @@
       <c r="A29" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="B29" s="14">
+      <c r="B29" s="15">
         <v>20.0</v>
       </c>
       <c r="C29" s="5"/>
@@ -4386,7 +4386,7 @@
       <c r="A30" s="10" t="s">
         <v>60</v>
       </c>
-      <c r="B30" s="14">
+      <c r="B30" s="15">
         <v>0.6</v>
       </c>
       <c r="C30" s="5"/>
@@ -4402,7 +4402,7 @@
       <c r="A31" s="10" t="s">
         <v>62</v>
       </c>
-      <c r="B31" s="14">
+      <c r="B31" s="15">
         <v>3.0</v>
       </c>
       <c r="C31" s="5"/>
@@ -4418,7 +4418,7 @@
       <c r="A32" s="10" t="s">
         <v>64</v>
       </c>
-      <c r="B32" s="14">
+      <c r="B32" s="15">
         <v>4.0</v>
       </c>
       <c r="C32" s="5"/>
@@ -4434,7 +4434,7 @@
       <c r="A33" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="B33" s="14">
+      <c r="B33" s="15">
         <v>2.0</v>
       </c>
       <c r="C33" s="5"/>
@@ -4450,7 +4450,7 @@
       <c r="A34" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="B34" s="14">
+      <c r="B34" s="15">
         <v>4.0</v>
       </c>
       <c r="C34" s="5"/>
@@ -4466,7 +4466,7 @@
       <c r="A35" s="10" t="s">
         <v>70</v>
       </c>
-      <c r="B35" s="14">
+      <c r="B35" s="15">
         <v>3.0</v>
       </c>
       <c r="C35" s="5"/>
@@ -14474,11 +14474,11 @@
       </c>
       <c r="B14" s="32">
         <f t="array" ref="B14">INDEX(Assumptions!$B$19:$D$19,B6)+Assumptions!$B$33*B9+Assumptions!$B$35*B10</f>
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C14" s="32">
         <f t="array" ref="C14">INDEX(Assumptions!$B$19:$D$19,C6)+Assumptions!$B$33*C9+Assumptions!$B$35*C10</f>
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="D14" s="32">
         <f t="array" ref="D14">INDEX(Assumptions!$B$19:$D$19,D6)+Assumptions!$B$33*D9+Assumptions!$B$35*D10</f>
@@ -14486,7 +14486,7 @@
       </c>
       <c r="E14" s="32">
         <f t="array" ref="E14">INDEX(Assumptions!$B$19:$D$19,E6)+Assumptions!$B$33*E9+Assumptions!$B$35*E10</f>
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="F14" s="5"/>
     </row>
@@ -14606,11 +14606,11 @@
       </c>
       <c r="B20" s="33">
         <f t="shared" ref="B20:E20" si="2">SUM(B14:B19)</f>
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="C20" s="33">
         <f t="shared" si="2"/>
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="D20" s="33">
         <f t="shared" si="2"/>
@@ -14618,7 +14618,7 @@
       </c>
       <c r="E20" s="33">
         <f t="shared" si="2"/>
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="F20" s="5"/>
     </row>
@@ -14646,19 +14646,19 @@
       </c>
       <c r="B23" s="34">
         <f>B14*Assumptions!$B$6</f>
-        <v>2200</v>
+        <v>3250</v>
       </c>
       <c r="C23" s="34">
         <f>C14*Assumptions!$B$6</f>
-        <v>6400</v>
+        <v>9000</v>
       </c>
       <c r="D23" s="34">
         <f>D14*Assumptions!$B$6</f>
-        <v>12400</v>
+        <v>15500</v>
       </c>
       <c r="E23" s="34">
         <f>E14*Assumptions!$B$6</f>
-        <v>6400</v>
+        <v>9000</v>
       </c>
       <c r="F23" s="5"/>
     </row>
@@ -14778,19 +14778,19 @@
       </c>
       <c r="B29" s="35">
         <f t="shared" ref="B29:E29" si="3">SUM(B23:B28)</f>
-        <v>10650</v>
+        <v>11700</v>
       </c>
       <c r="C29" s="35">
         <f t="shared" si="3"/>
-        <v>19150</v>
+        <v>21750</v>
       </c>
       <c r="D29" s="35">
         <f t="shared" si="3"/>
-        <v>31050</v>
+        <v>34150</v>
       </c>
       <c r="E29" s="35">
         <f t="shared" si="3"/>
-        <v>19150</v>
+        <v>21750</v>
       </c>
       <c r="F29" s="5"/>
     </row>
@@ -14808,11 +14808,11 @@
       </c>
       <c r="D30" s="34">
         <f>D11*Assumptions!$B$12</f>
-        <v>7000</v>
+        <v>6000</v>
       </c>
       <c r="E30" s="34">
         <f>E11*Assumptions!$B$12</f>
-        <v>3500</v>
+        <v>3000</v>
       </c>
       <c r="F30" s="5"/>
     </row>
@@ -14822,19 +14822,19 @@
       </c>
       <c r="B31" s="35">
         <f t="shared" ref="B31:E31" si="4">B29+B30</f>
-        <v>10650</v>
+        <v>11700</v>
       </c>
       <c r="C31" s="35">
         <f t="shared" si="4"/>
-        <v>19150</v>
+        <v>21750</v>
       </c>
       <c r="D31" s="35">
         <f t="shared" si="4"/>
-        <v>38050</v>
+        <v>40150</v>
       </c>
       <c r="E31" s="35">
         <f t="shared" si="4"/>
-        <v>22650</v>
+        <v>24750</v>
       </c>
       <c r="F31" s="5"/>
     </row>
@@ -14844,19 +14844,19 @@
       </c>
       <c r="B32" s="35">
         <f>CEILING(B31,Assumptions!$B$13)</f>
-        <v>10700</v>
+        <v>11700</v>
       </c>
       <c r="C32" s="35">
         <f>CEILING(C31,Assumptions!$B$13)</f>
-        <v>19200</v>
+        <v>21800</v>
       </c>
       <c r="D32" s="35">
         <f>CEILING(D31,Assumptions!$B$13)</f>
-        <v>38100</v>
+        <v>40200</v>
       </c>
       <c r="E32" s="35">
         <f>CEILING(E31,Assumptions!$B$13)</f>
-        <v>22700</v>
+        <v>24800</v>
       </c>
       <c r="F32" s="5"/>
     </row>
@@ -14932,7 +14932,7 @@
       </c>
       <c r="E38" s="42">
         <f t="shared" ref="E38:E40" si="5">INDEX($B$32:$E$32,MATCH(D38,$B$4:$E$4,0))</f>
-        <v>10700</v>
+        <v>11700</v>
       </c>
       <c r="F38" s="5"/>
     </row>
@@ -14954,7 +14954,7 @@
       </c>
       <c r="E39" s="42">
         <f t="shared" si="5"/>
-        <v>19200</v>
+        <v>21800</v>
       </c>
       <c r="F39" s="5"/>
     </row>
@@ -14976,7 +14976,7 @@
       </c>
       <c r="E40" s="42">
         <f t="shared" si="5"/>
-        <v>38100</v>
+        <v>40200</v>
       </c>
       <c r="F40" s="5"/>
     </row>
@@ -14989,7 +14989,7 @@
       <c r="D41" s="18"/>
       <c r="E41" s="43">
         <f>SUM(E38:E40)</f>
-        <v>68000</v>
+        <v>73700</v>
       </c>
       <c r="F41" s="5"/>
     </row>

</xml_diff>